<commit_message>
Add orders 105852 to unified Nova America spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Nova_America_Unificado.xlsx
+++ b/pedidos/Pedidos_Nova_America_Unificado.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V43"/>
+  <dimension ref="A1:V50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1714,7 +1714,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>105844</v>
+        <v>105852</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1722,57 +1722,42 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>99069557</v>
+        <v>947706</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AFB130</t>
+          <t>LMM004</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AFB130TC</t>
+          <t>LMM004BG</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AFB130TC</t>
+          <t>LMM004BG</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>114.1</v>
+        <v>17.51</v>
       </c>
       <c r="H24" t="n">
         <v>1</v>
       </c>
-      <c r="M24" t="n">
-        <v>1</v>
-      </c>
-      <c r="N24" t="n">
-        <v>2</v>
-      </c>
-      <c r="O24" t="n">
-        <v>2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>2</v>
-      </c>
-      <c r="R24" t="n">
-        <v>1</v>
+      <c r="T24" t="n">
+        <v>24</v>
       </c>
       <c r="U24" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="V24" t="n">
-        <v>1369.2</v>
+        <v>420.24</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>105844</v>
+        <v>105852</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1780,60 +1765,42 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21043</v>
+        <v>939642</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ASF711</t>
+          <t>LMM004</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ASF711CF</t>
+          <t>LMM004MM</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>ASF711CF</t>
+          <t>LMM004MM</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>74.66</v>
+        <v>17.51</v>
       </c>
       <c r="H25" t="n">
         <v>1</v>
       </c>
-      <c r="M25" t="n">
-        <v>1</v>
-      </c>
-      <c r="N25" t="n">
-        <v>2</v>
-      </c>
-      <c r="O25" t="n">
-        <v>3</v>
-      </c>
-      <c r="P25" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>3</v>
-      </c>
-      <c r="R25" t="n">
-        <v>2</v>
-      </c>
-      <c r="S25" t="n">
-        <v>1</v>
+      <c r="T25" t="n">
+        <v>24</v>
       </c>
       <c r="U25" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="V25" t="n">
-        <v>1119.9</v>
+        <v>420.24</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>105844</v>
+        <v>105852</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1841,57 +1808,42 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>62522833</v>
+        <v>939643</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SLB034</t>
+          <t>LMM004</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SLB034PT</t>
+          <t>LMM004PT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SLB034PT</t>
+          <t>LMM004PT</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>200.54</v>
+        <v>17.51</v>
       </c>
       <c r="H26" t="n">
         <v>1</v>
       </c>
-      <c r="N26" t="n">
-        <v>2</v>
-      </c>
-      <c r="O26" t="n">
-        <v>3</v>
-      </c>
-      <c r="P26" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>4</v>
-      </c>
-      <c r="R26" t="n">
-        <v>3</v>
-      </c>
-      <c r="S26" t="n">
-        <v>2</v>
+      <c r="T26" t="n">
+        <v>36</v>
       </c>
       <c r="U26" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="V26" t="n">
-        <v>3609.72</v>
+        <v>630.36</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>105844</v>
+        <v>105852</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1899,60 +1851,42 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>164567877</v>
+        <v>21174</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SLB034</t>
+          <t>LMM009</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SLB034TN</t>
+          <t>LMM009PT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SLB034TN</t>
+          <t>LMM009PT</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>200.54</v>
+        <v>15.63</v>
       </c>
       <c r="H27" t="n">
         <v>1</v>
       </c>
-      <c r="M27" t="n">
-        <v>1</v>
-      </c>
-      <c r="N27" t="n">
-        <v>1</v>
-      </c>
-      <c r="O27" t="n">
-        <v>4</v>
-      </c>
-      <c r="P27" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>3</v>
-      </c>
-      <c r="R27" t="n">
-        <v>1</v>
-      </c>
-      <c r="S27" t="n">
-        <v>1</v>
+      <c r="T27" t="n">
+        <v>36</v>
       </c>
       <c r="U27" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="V27" t="n">
-        <v>3008.1</v>
+        <v>562.6799999999999</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>105844</v>
+        <v>105852</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1960,60 +1894,42 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>179157149</v>
+        <v>79775189</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SWL134</t>
+          <t>LMM619</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SWL134CF</t>
+          <t>LMM619BC</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>SWL134CF</t>
+          <t>LMM619BC</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>183.09</v>
+        <v>15.33</v>
       </c>
       <c r="H28" t="n">
         <v>1</v>
       </c>
-      <c r="M28" t="n">
-        <v>1</v>
-      </c>
-      <c r="N28" t="n">
-        <v>2</v>
-      </c>
-      <c r="O28" t="n">
-        <v>3</v>
-      </c>
-      <c r="P28" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>2</v>
-      </c>
-      <c r="R28" t="n">
-        <v>2</v>
-      </c>
-      <c r="S28" t="n">
-        <v>1</v>
+      <c r="T28" t="n">
+        <v>60</v>
       </c>
       <c r="U28" t="n">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="V28" t="n">
-        <v>2563.26</v>
+        <v>919.8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>105844</v>
+        <v>105852</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2021,57 +1937,42 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>226799445</v>
+        <v>79775190</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>WSCR57</t>
+          <t>LMM619</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WSCR57BI</t>
+          <t>LMM619BG</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>WSCR57BI</t>
+          <t>LMM619BG</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>159.25</v>
+        <v>15.33</v>
       </c>
       <c r="H29" t="n">
         <v>1</v>
       </c>
-      <c r="I29" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" t="n">
-        <v>3</v>
-      </c>
-      <c r="K29" t="n">
-        <v>4</v>
-      </c>
-      <c r="L29" t="n">
-        <v>4</v>
-      </c>
-      <c r="M29" t="n">
-        <v>2</v>
-      </c>
-      <c r="N29" t="n">
-        <v>1</v>
+      <c r="T29" t="n">
+        <v>36</v>
       </c>
       <c r="U29" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="V29" t="n">
-        <v>2388.75</v>
+        <v>551.88</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>105844</v>
+        <v>105852</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2079,57 +1980,42 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>226799459</v>
+        <v>79775193</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>WSCR89</t>
+          <t>LMM619</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WSCR89TN</t>
+          <t>LMM619PT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>WSCR89TN</t>
+          <t>LMM619PT</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>161.58</v>
+        <v>15.33</v>
       </c>
       <c r="H30" t="n">
         <v>1</v>
       </c>
-      <c r="I30" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" t="n">
-        <v>3</v>
-      </c>
-      <c r="K30" t="n">
-        <v>4</v>
-      </c>
-      <c r="L30" t="n">
-        <v>4</v>
-      </c>
-      <c r="M30" t="n">
-        <v>2</v>
-      </c>
-      <c r="N30" t="n">
-        <v>1</v>
+      <c r="T30" t="n">
+        <v>60</v>
       </c>
       <c r="U30" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="V30" t="n">
-        <v>2423.7</v>
+        <v>919.8</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>105845</v>
+        <v>105844</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2137,25 +2023,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>227068437</v>
+        <v>99069557</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>SAF126</t>
+          <t>AFB130</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SAF126BK</t>
+          <t>AFB130TC</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>SAF126BK</t>
+          <t>AFB130TC</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>135.3</v>
+        <v>114.1</v>
       </c>
       <c r="H31" t="n">
         <v>1</v>
@@ -2164,33 +2050,30 @@
         <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P31" t="n">
         <v>4</v>
       </c>
       <c r="Q31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R31" t="n">
-        <v>2</v>
-      </c>
-      <c r="S31" t="n">
         <v>1</v>
       </c>
       <c r="U31" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="V31" t="n">
-        <v>2435.4</v>
+        <v>1369.2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>105845</v>
+        <v>105844</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2198,25 +2081,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>194597523</v>
+        <v>21043</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SRF025</t>
+          <t>ASF711</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SRF025MR</t>
+          <t>ASF711CF</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>SRF025MR</t>
+          <t>ASF711CF</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>153.55</v>
+        <v>74.66</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
@@ -2225,7 +2108,7 @@
         <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O32" t="n">
         <v>3</v>
@@ -2234,7 +2117,7 @@
         <v>3</v>
       </c>
       <c r="Q32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R32" t="n">
         <v>2</v>
@@ -2246,12 +2129,12 @@
         <v>15</v>
       </c>
       <c r="V32" t="n">
-        <v>2303.25</v>
+        <v>1119.9</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>105845</v>
+        <v>105844</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2259,60 +2142,57 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>226787944</v>
+        <v>62522833</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SRT028</t>
+          <t>SLB034</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SRT028BK</t>
+          <t>SLB034PT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>SRT028BK</t>
+          <t>SLB034PT</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>159.78</v>
+        <v>200.54</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
       </c>
-      <c r="M33" t="n">
-        <v>1</v>
-      </c>
       <c r="N33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P33" t="n">
         <v>4</v>
       </c>
       <c r="Q33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U33" t="n">
         <v>18</v>
       </c>
       <c r="V33" t="n">
-        <v>2876.04</v>
+        <v>3609.72</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>105845</v>
+        <v>105844</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2320,25 +2200,25 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>160831013</v>
+        <v>164567877</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SVS027</t>
+          <t>SLB034</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SVS027CM</t>
+          <t>SLB034TN</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>SVS027CM</t>
+          <t>SLB034TN</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>145.11</v>
+        <v>200.54</v>
       </c>
       <c r="H34" t="n">
         <v>1</v>
@@ -2347,27 +2227,33 @@
         <v>1</v>
       </c>
       <c r="N34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q34" t="n">
         <v>3</v>
       </c>
+      <c r="R34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" t="n">
+        <v>1</v>
+      </c>
       <c r="U34" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="V34" t="n">
-        <v>1741.32</v>
+        <v>3008.1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>105845</v>
+        <v>105844</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2375,57 +2261,60 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>99645682</v>
+        <v>179157149</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>WSC003</t>
+          <t>SWL134</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WSC003OW</t>
+          <t>SWL134CF</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>WSC003OW</t>
+          <t>SWL134CF</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>138.2</v>
+        <v>183.09</v>
       </c>
       <c r="H35" t="n">
         <v>1</v>
       </c>
-      <c r="I35" t="n">
-        <v>1</v>
-      </c>
-      <c r="J35" t="n">
-        <v>1</v>
-      </c>
-      <c r="K35" t="n">
-        <v>4</v>
-      </c>
-      <c r="L35" t="n">
-        <v>5</v>
-      </c>
       <c r="M35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
+        <v>2</v>
+      </c>
+      <c r="O35" t="n">
+        <v>3</v>
+      </c>
+      <c r="P35" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>2</v>
+      </c>
+      <c r="R35" t="n">
+        <v>2</v>
+      </c>
+      <c r="S35" t="n">
         <v>1</v>
       </c>
       <c r="U35" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V35" t="n">
-        <v>2073</v>
+        <v>2563.26</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>105851</v>
+        <v>105844</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2433,42 +2322,57 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>13222</v>
+        <v>226799445</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>HCT173</t>
+          <t>WSCR57</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>HCT173CF</t>
+          <t>WSCR57BI</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>HCT173CF</t>
+          <t>WSCR57BI</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>52.89</v>
+        <v>159.25</v>
       </c>
       <c r="H36" t="n">
         <v>1</v>
       </c>
-      <c r="T36" t="n">
-        <v>9</v>
+      <c r="I36" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" t="n">
+        <v>3</v>
+      </c>
+      <c r="K36" t="n">
+        <v>4</v>
+      </c>
+      <c r="L36" t="n">
+        <v>4</v>
+      </c>
+      <c r="M36" t="n">
+        <v>2</v>
+      </c>
+      <c r="N36" t="n">
+        <v>1</v>
       </c>
       <c r="U36" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="V36" t="n">
-        <v>476.01</v>
+        <v>2388.75</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>105851</v>
+        <v>105844</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2476,42 +2380,57 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>13223</v>
+        <v>226799459</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>HCT173</t>
+          <t>WSCR89</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>HCT173PT</t>
+          <t>WSCR89TN</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>HCT173PT</t>
+          <t>WSCR89TN</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>52.89</v>
+        <v>161.58</v>
       </c>
       <c r="H37" t="n">
         <v>1</v>
       </c>
-      <c r="T37" t="n">
-        <v>6</v>
+      <c r="I37" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" t="n">
+        <v>4</v>
+      </c>
+      <c r="L37" t="n">
+        <v>4</v>
+      </c>
+      <c r="M37" t="n">
+        <v>2</v>
+      </c>
+      <c r="N37" t="n">
+        <v>1</v>
       </c>
       <c r="U37" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="V37" t="n">
-        <v>317.34</v>
+        <v>2423.7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>105851</v>
+        <v>105845</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2519,42 +2438,60 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>138654477</v>
+        <v>227068437</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>MCC008</t>
+          <t>SAF126</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>MCC008TN</t>
+          <t>SAF126BK</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>MCC008TN</t>
+          <t>SAF126BK</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>39.04</v>
+        <v>135.3</v>
       </c>
       <c r="H38" t="n">
         <v>1</v>
       </c>
-      <c r="T38" t="n">
-        <v>9</v>
+      <c r="M38" t="n">
+        <v>1</v>
+      </c>
+      <c r="N38" t="n">
+        <v>3</v>
+      </c>
+      <c r="O38" t="n">
+        <v>4</v>
+      </c>
+      <c r="P38" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>3</v>
+      </c>
+      <c r="R38" t="n">
+        <v>2</v>
+      </c>
+      <c r="S38" t="n">
+        <v>1</v>
       </c>
       <c r="U38" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="V38" t="n">
-        <v>351.36</v>
+        <v>2435.4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>105851</v>
+        <v>105845</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2562,42 +2499,60 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>138654478</v>
+        <v>194597523</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>MCC008</t>
+          <t>SRF025</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>MCC008VR</t>
+          <t>SRF025MR</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>MCC008VR</t>
+          <t>SRF025MR</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>39.04</v>
+        <v>153.55</v>
       </c>
       <c r="H39" t="n">
         <v>1</v>
       </c>
-      <c r="T39" t="n">
-        <v>9</v>
+      <c r="M39" t="n">
+        <v>1</v>
+      </c>
+      <c r="N39" t="n">
+        <v>3</v>
+      </c>
+      <c r="O39" t="n">
+        <v>3</v>
+      </c>
+      <c r="P39" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>2</v>
+      </c>
+      <c r="R39" t="n">
+        <v>2</v>
+      </c>
+      <c r="S39" t="n">
+        <v>1</v>
       </c>
       <c r="U39" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="V39" t="n">
-        <v>351.36</v>
+        <v>2303.25</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>105856</v>
+        <v>105845</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2605,57 +2560,60 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>178969123</v>
+        <v>226787944</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>PRA127</t>
+          <t>SRT028</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>PRA127CF</t>
+          <t>SRT028BK</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>PRA127CF</t>
+          <t>SRT028BK</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>61.13</v>
+        <v>159.78</v>
       </c>
       <c r="H40" t="n">
         <v>1</v>
       </c>
-      <c r="I40" t="n">
-        <v>1</v>
-      </c>
-      <c r="J40" t="n">
-        <v>3</v>
-      </c>
-      <c r="K40" t="n">
+      <c r="M40" t="n">
+        <v>1</v>
+      </c>
+      <c r="N40" t="n">
+        <v>3</v>
+      </c>
+      <c r="O40" t="n">
         <v>4</v>
       </c>
-      <c r="L40" t="n">
-        <v>3</v>
-      </c>
-      <c r="M40" t="n">
-        <v>3</v>
-      </c>
-      <c r="N40" t="n">
+      <c r="P40" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>3</v>
+      </c>
+      <c r="R40" t="n">
+        <v>2</v>
+      </c>
+      <c r="S40" t="n">
         <v>1</v>
       </c>
       <c r="U40" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="V40" t="n">
-        <v>916.95</v>
+        <v>2876.04</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>105856</v>
+        <v>105845</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -2663,57 +2621,54 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>226774175</v>
+        <v>160831013</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>PRA728</t>
+          <t>SVS027</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>PRA728FD</t>
+          <t>SVS027CM</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PRA728FD</t>
+          <t>SVS027CM</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>70.93000000000001</v>
+        <v>145.11</v>
       </c>
       <c r="H41" t="n">
         <v>1</v>
       </c>
-      <c r="I41" t="n">
-        <v>1</v>
-      </c>
-      <c r="J41" t="n">
-        <v>3</v>
-      </c>
-      <c r="K41" t="n">
-        <v>4</v>
-      </c>
-      <c r="L41" t="n">
-        <v>3</v>
-      </c>
       <c r="M41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="O41" t="n">
+        <v>3</v>
+      </c>
+      <c r="P41" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>3</v>
       </c>
       <c r="U41" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="V41" t="n">
-        <v>1063.95</v>
+        <v>1741.32</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>105856</v>
+        <v>105845</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2721,25 +2676,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>226774176</v>
+        <v>99645682</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>PRA728</t>
+          <t>WSC003</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>PRA728VO</t>
+          <t>WSC003OW</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>PRA728VO</t>
+          <t>WSC003OW</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>70.93000000000001</v>
+        <v>138.2</v>
       </c>
       <c r="H42" t="n">
         <v>1</v>
@@ -2748,82 +2703,428 @@
         <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N42" t="n">
         <v>1</v>
       </c>
       <c r="U42" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="V42" t="n">
-        <v>851.16</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
+        <v>105851</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>13222</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>HCT173</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>HCT173CF</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>HCT173CF</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>52.89</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1</v>
+      </c>
+      <c r="T43" t="n">
+        <v>9</v>
+      </c>
+      <c r="U43" t="n">
+        <v>9</v>
+      </c>
+      <c r="V43" t="n">
+        <v>476.01</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>105851</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>13223</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>HCT173</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>HCT173PT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>HCT173PT</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>52.89</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1</v>
+      </c>
+      <c r="T44" t="n">
+        <v>6</v>
+      </c>
+      <c r="U44" t="n">
+        <v>6</v>
+      </c>
+      <c r="V44" t="n">
+        <v>317.34</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>105851</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>138654477</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>MCC008</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>MCC008TN</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>MCC008TN</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>39.04</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1</v>
+      </c>
+      <c r="T45" t="n">
+        <v>9</v>
+      </c>
+      <c r="U45" t="n">
+        <v>9</v>
+      </c>
+      <c r="V45" t="n">
+        <v>351.36</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>105851</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>138654478</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>MCC008</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>MCC008VR</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>MCC008VR</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>39.04</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1</v>
+      </c>
+      <c r="T46" t="n">
+        <v>9</v>
+      </c>
+      <c r="U46" t="n">
+        <v>9</v>
+      </c>
+      <c r="V46" t="n">
+        <v>351.36</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
         <v>105856</v>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>SH. NOVA AMERICA</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>178969123</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PRA127</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>PRA127CF</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>PRA127CF</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>61.13</v>
+      </c>
+      <c r="H47" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K47" t="n">
+        <v>4</v>
+      </c>
+      <c r="L47" t="n">
+        <v>3</v>
+      </c>
+      <c r="M47" t="n">
+        <v>3</v>
+      </c>
+      <c r="N47" t="n">
+        <v>1</v>
+      </c>
+      <c r="U47" t="n">
+        <v>15</v>
+      </c>
+      <c r="V47" t="n">
+        <v>916.95</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>105856</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>226774175</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>PRA728</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>PRA728FD</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>PRA728FD</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="H48" t="n">
+        <v>1</v>
+      </c>
+      <c r="I48" t="n">
+        <v>1</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" t="n">
+        <v>4</v>
+      </c>
+      <c r="L48" t="n">
+        <v>3</v>
+      </c>
+      <c r="M48" t="n">
+        <v>3</v>
+      </c>
+      <c r="N48" t="n">
+        <v>1</v>
+      </c>
+      <c r="U48" t="n">
+        <v>15</v>
+      </c>
+      <c r="V48" t="n">
+        <v>1063.95</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>105856</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>226774176</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>PRA728</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>PRA728VO</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>PRA728VO</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" t="n">
+        <v>3</v>
+      </c>
+      <c r="L49" t="n">
+        <v>3</v>
+      </c>
+      <c r="M49" t="n">
+        <v>2</v>
+      </c>
+      <c r="N49" t="n">
+        <v>1</v>
+      </c>
+      <c r="U49" t="n">
+        <v>12</v>
+      </c>
+      <c r="V49" t="n">
+        <v>851.16</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>105856</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
         <v>226799120</v>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>TBC207</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>TBC207CA</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>TBC207CA</t>
         </is>
       </c>
-      <c r="G43" t="n">
+      <c r="G50" t="n">
         <v>56.96</v>
       </c>
-      <c r="H43" t="n">
-        <v>1</v>
-      </c>
-      <c r="I43" t="n">
-        <v>1</v>
-      </c>
-      <c r="J43" t="n">
-        <v>3</v>
-      </c>
-      <c r="K43" t="n">
+      <c r="H50" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" t="n">
+        <v>1</v>
+      </c>
+      <c r="J50" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" t="n">
         <v>5</v>
       </c>
-      <c r="L43" t="n">
+      <c r="L50" t="n">
         <v>4</v>
       </c>
-      <c r="M43" t="n">
-        <v>3</v>
-      </c>
-      <c r="N43" t="n">
-        <v>2</v>
-      </c>
-      <c r="U43" t="n">
+      <c r="M50" t="n">
+        <v>3</v>
+      </c>
+      <c r="N50" t="n">
+        <v>2</v>
+      </c>
+      <c r="U50" t="n">
         <v>18</v>
       </c>
-      <c r="V43" t="n">
+      <c r="V50" t="n">
         <v>1025.28</v>
       </c>
     </row>
@@ -3113,15 +3414,26 @@
           <t>PRIMAR IND TEXTIL LTDA</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>N2_RelB2bCarrinhoExcel-18h46.xlsx</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEM ARQUIVO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>276</v>
       </c>
+      <c r="G8" t="n">
+        <v>276</v>
+      </c>
       <c r="H8" t="n">
+        <v>4425</v>
+      </c>
+      <c r="I8" t="n">
         <v>4425</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add order 105849 to unified Nova America spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Nova_America_Unificado.xlsx
+++ b/pedidos/Pedidos_Nova_America_Unificado.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V50"/>
+  <dimension ref="A1:V66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2015,7 +2015,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>105844</v>
+        <v>105849</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2023,57 +2023,42 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>99069557</v>
+        <v>226773022</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>AFB130</t>
+          <t>GBF191</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AFB130TC</t>
+          <t>GBF191CF</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AFB130TC</t>
+          <t>GBF191CF</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>114.1</v>
+        <v>242.99</v>
       </c>
       <c r="H31" t="n">
         <v>1</v>
       </c>
-      <c r="M31" t="n">
-        <v>1</v>
-      </c>
-      <c r="N31" t="n">
-        <v>2</v>
-      </c>
-      <c r="O31" t="n">
-        <v>2</v>
-      </c>
-      <c r="P31" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>2</v>
-      </c>
-      <c r="R31" t="n">
-        <v>1</v>
+      <c r="T31" t="n">
+        <v>2</v>
       </c>
       <c r="U31" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="V31" t="n">
-        <v>1369.2</v>
+        <v>485.98</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>105844</v>
+        <v>105849</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2081,60 +2066,42 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>21043</v>
+        <v>226773023</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>ASF711</t>
+          <t>GBF191</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ASF711CF</t>
+          <t>GBF191VO</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ASF711CF</t>
+          <t>GBF191VO</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>74.66</v>
+        <v>242.99</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
       </c>
-      <c r="M32" t="n">
-        <v>1</v>
-      </c>
-      <c r="N32" t="n">
-        <v>2</v>
-      </c>
-      <c r="O32" t="n">
-        <v>3</v>
-      </c>
-      <c r="P32" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>3</v>
-      </c>
-      <c r="R32" t="n">
-        <v>2</v>
-      </c>
-      <c r="S32" t="n">
-        <v>1</v>
+      <c r="T32" t="n">
+        <v>2</v>
       </c>
       <c r="U32" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="V32" t="n">
-        <v>1119.9</v>
+        <v>485.98</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>105844</v>
+        <v>105849</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2142,57 +2109,42 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>62522833</v>
+        <v>226773071</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SLB034</t>
+          <t>GBF269</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SLB034PT</t>
+          <t>GBF269FD</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>SLB034PT</t>
+          <t>GBF269FD</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>200.54</v>
+        <v>235</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
       </c>
-      <c r="N33" t="n">
-        <v>2</v>
-      </c>
-      <c r="O33" t="n">
-        <v>3</v>
-      </c>
-      <c r="P33" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>4</v>
-      </c>
-      <c r="R33" t="n">
-        <v>3</v>
-      </c>
-      <c r="S33" t="n">
+      <c r="T33" t="n">
         <v>2</v>
       </c>
       <c r="U33" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="V33" t="n">
-        <v>3609.72</v>
+        <v>470</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>105844</v>
+        <v>105849</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2200,60 +2152,42 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>164567877</v>
+        <v>218687255</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SLB034</t>
+          <t>GBF445</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SLB034TN</t>
+          <t>GBF445CF</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>SLB034TN</t>
+          <t>GBF445CF</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>200.54</v>
+        <v>122.67</v>
       </c>
       <c r="H34" t="n">
         <v>1</v>
       </c>
-      <c r="M34" t="n">
-        <v>1</v>
-      </c>
-      <c r="N34" t="n">
-        <v>1</v>
-      </c>
-      <c r="O34" t="n">
-        <v>4</v>
-      </c>
-      <c r="P34" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>3</v>
-      </c>
-      <c r="R34" t="n">
-        <v>1</v>
-      </c>
-      <c r="S34" t="n">
-        <v>1</v>
+      <c r="T34" t="n">
+        <v>2</v>
       </c>
       <c r="U34" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="V34" t="n">
-        <v>3008.1</v>
+        <v>245.34</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>105844</v>
+        <v>105849</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2261,60 +2195,42 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>179157149</v>
+        <v>58174815</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SWL134</t>
+          <t>GBF445</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SWL134CF</t>
+          <t>GBF445PT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>SWL134CF</t>
+          <t>GBF445PT</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>183.09</v>
+        <v>122.67</v>
       </c>
       <c r="H35" t="n">
         <v>1</v>
       </c>
-      <c r="M35" t="n">
-        <v>1</v>
-      </c>
-      <c r="N35" t="n">
-        <v>2</v>
-      </c>
-      <c r="O35" t="n">
-        <v>3</v>
-      </c>
-      <c r="P35" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>2</v>
-      </c>
-      <c r="R35" t="n">
-        <v>2</v>
-      </c>
-      <c r="S35" t="n">
-        <v>1</v>
+      <c r="T35" t="n">
+        <v>3</v>
       </c>
       <c r="U35" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="V35" t="n">
-        <v>2563.26</v>
+        <v>368.01</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>105844</v>
+        <v>105849</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2322,57 +2238,42 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>226799445</v>
+        <v>226773215</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>WSCR57</t>
+          <t>GBF786</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WSCR57BI</t>
+          <t>GBF786CF</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>WSCR57BI</t>
+          <t>GBF786CF</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>159.25</v>
+        <v>200.69</v>
       </c>
       <c r="H36" t="n">
         <v>1</v>
       </c>
-      <c r="I36" t="n">
-        <v>1</v>
-      </c>
-      <c r="J36" t="n">
-        <v>3</v>
-      </c>
-      <c r="K36" t="n">
-        <v>4</v>
-      </c>
-      <c r="L36" t="n">
-        <v>4</v>
-      </c>
-      <c r="M36" t="n">
-        <v>2</v>
-      </c>
-      <c r="N36" t="n">
-        <v>1</v>
+      <c r="T36" t="n">
+        <v>2</v>
       </c>
       <c r="U36" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="V36" t="n">
-        <v>2388.75</v>
+        <v>401.38</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>105844</v>
+        <v>105849</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2380,57 +2281,42 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>226799459</v>
+        <v>226773217</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>WSCR89</t>
+          <t>GBF788</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WSCR89TN</t>
+          <t>GBF788PT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>WSCR89TN</t>
+          <t>GBF788PT</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>161.58</v>
+        <v>138.06</v>
       </c>
       <c r="H37" t="n">
         <v>1</v>
       </c>
-      <c r="I37" t="n">
-        <v>1</v>
-      </c>
-      <c r="J37" t="n">
-        <v>3</v>
-      </c>
-      <c r="K37" t="n">
-        <v>4</v>
-      </c>
-      <c r="L37" t="n">
-        <v>4</v>
-      </c>
-      <c r="M37" t="n">
-        <v>2</v>
-      </c>
-      <c r="N37" t="n">
-        <v>1</v>
+      <c r="T37" t="n">
+        <v>3</v>
       </c>
       <c r="U37" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="V37" t="n">
-        <v>2423.7</v>
+        <v>414.18</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>105845</v>
+        <v>105849</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2438,60 +2324,42 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>227068437</v>
+        <v>226773218</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>SAF126</t>
+          <t>GBF788</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SAF126BK</t>
+          <t>GBF788TN</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>SAF126BK</t>
+          <t>GBF788TN</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>135.3</v>
+        <v>138.06</v>
       </c>
       <c r="H38" t="n">
         <v>1</v>
       </c>
-      <c r="M38" t="n">
-        <v>1</v>
-      </c>
-      <c r="N38" t="n">
-        <v>3</v>
-      </c>
-      <c r="O38" t="n">
-        <v>4</v>
-      </c>
-      <c r="P38" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>3</v>
-      </c>
-      <c r="R38" t="n">
-        <v>2</v>
-      </c>
-      <c r="S38" t="n">
-        <v>1</v>
+      <c r="T38" t="n">
+        <v>3</v>
       </c>
       <c r="U38" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="V38" t="n">
-        <v>2435.4</v>
+        <v>414.18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>105845</v>
+        <v>105849</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2499,60 +2367,42 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>194597523</v>
+        <v>177646295</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SRF025</t>
+          <t>GBF827</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SRF025MR</t>
+          <t>GBF827PT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>SRF025MR</t>
+          <t>GBF827PT</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>153.55</v>
+        <v>85.78</v>
       </c>
       <c r="H39" t="n">
         <v>1</v>
       </c>
-      <c r="M39" t="n">
-        <v>1</v>
-      </c>
-      <c r="N39" t="n">
-        <v>3</v>
-      </c>
-      <c r="O39" t="n">
-        <v>3</v>
-      </c>
-      <c r="P39" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>2</v>
-      </c>
-      <c r="R39" t="n">
-        <v>2</v>
-      </c>
-      <c r="S39" t="n">
-        <v>1</v>
+      <c r="T39" t="n">
+        <v>8</v>
       </c>
       <c r="U39" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="V39" t="n">
-        <v>2303.25</v>
+        <v>686.24</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>105845</v>
+        <v>105849</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2560,60 +2410,42 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>226787944</v>
+        <v>137476322</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>SRT028</t>
+          <t>GSN810</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SRT028BK</t>
+          <t>GSN810PT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>SRT028BK</t>
+          <t>GSN810PT</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>159.78</v>
+        <v>122.2</v>
       </c>
       <c r="H40" t="n">
         <v>1</v>
       </c>
-      <c r="M40" t="n">
-        <v>1</v>
-      </c>
-      <c r="N40" t="n">
-        <v>3</v>
-      </c>
-      <c r="O40" t="n">
-        <v>4</v>
-      </c>
-      <c r="P40" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>3</v>
-      </c>
-      <c r="R40" t="n">
-        <v>2</v>
-      </c>
-      <c r="S40" t="n">
-        <v>1</v>
+      <c r="T40" t="n">
+        <v>2</v>
       </c>
       <c r="U40" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="V40" t="n">
-        <v>2876.04</v>
+        <v>244.4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>105845</v>
+        <v>105849</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -2621,54 +2453,42 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>160831013</v>
+        <v>147957944</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>SVS027</t>
+          <t>GSN811</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SVS027CM</t>
+          <t>GSN811PT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>SVS027CM</t>
+          <t>GSN811PT</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>145.11</v>
+        <v>123.38</v>
       </c>
       <c r="H41" t="n">
         <v>1</v>
       </c>
-      <c r="M41" t="n">
-        <v>1</v>
-      </c>
-      <c r="N41" t="n">
-        <v>2</v>
-      </c>
-      <c r="O41" t="n">
-        <v>3</v>
-      </c>
-      <c r="P41" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>3</v>
+      <c r="T41" t="n">
+        <v>4</v>
       </c>
       <c r="U41" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="V41" t="n">
-        <v>1741.32</v>
+        <v>493.52</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>105845</v>
+        <v>105849</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2676,57 +2496,42 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>99645682</v>
+        <v>147957945</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>WSC003</t>
+          <t>GSN811</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>WSC003OW</t>
+          <t>GSN811TN</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>WSC003OW</t>
+          <t>GSN811TN</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>138.2</v>
+        <v>123.38</v>
       </c>
       <c r="H42" t="n">
         <v>1</v>
       </c>
-      <c r="I42" t="n">
-        <v>1</v>
-      </c>
-      <c r="J42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" t="n">
+      <c r="T42" t="n">
         <v>4</v>
       </c>
-      <c r="L42" t="n">
-        <v>5</v>
-      </c>
-      <c r="M42" t="n">
-        <v>3</v>
-      </c>
-      <c r="N42" t="n">
-        <v>1</v>
-      </c>
       <c r="U42" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="V42" t="n">
-        <v>2073</v>
+        <v>493.52</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>105851</v>
+        <v>105849</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2734,42 +2539,42 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>13222</v>
+        <v>16652</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>HCT173</t>
+          <t>HCT054</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>HCT173CF</t>
+          <t>HCT054CF</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>HCT173CF</t>
+          <t>HCT054CF</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>52.89</v>
+        <v>45.77</v>
       </c>
       <c r="H43" t="n">
         <v>1</v>
       </c>
       <c r="T43" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="U43" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="V43" t="n">
-        <v>476.01</v>
+        <v>183.08</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>105851</v>
+        <v>105849</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2777,42 +2582,42 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>13223</v>
+        <v>16653</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>HCT173</t>
+          <t>HCT054</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>HCT173PT</t>
+          <t>HCT054PT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>HCT173PT</t>
+          <t>HCT054PT</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>52.89</v>
+        <v>45.77</v>
       </c>
       <c r="H44" t="n">
         <v>1</v>
       </c>
       <c r="T44" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="U44" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="V44" t="n">
-        <v>317.34</v>
+        <v>411.93</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>105851</v>
+        <v>105849</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2820,25 +2625,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>138654477</v>
+        <v>10222949</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>MCC008</t>
+          <t>HCT095</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>MCC008TN</t>
+          <t>HCT095PT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>MCC008TN</t>
+          <t>HCT095PT</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>39.04</v>
+        <v>49.35</v>
       </c>
       <c r="H45" t="n">
         <v>1</v>
@@ -2850,12 +2655,12 @@
         <v>9</v>
       </c>
       <c r="V45" t="n">
-        <v>351.36</v>
+        <v>444.15</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>105851</v>
+        <v>105849</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2863,42 +2668,42 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>138654478</v>
+        <v>10222951</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>MCC008</t>
+          <t>HCT096</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>MCC008VR</t>
+          <t>HCT096PT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>MCC008VR</t>
+          <t>HCT096PT</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>39.04</v>
+        <v>45.78</v>
       </c>
       <c r="H46" t="n">
         <v>1</v>
       </c>
       <c r="T46" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="U46" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="V46" t="n">
-        <v>351.36</v>
+        <v>274.68</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>105856</v>
+        <v>105844</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2906,57 +2711,57 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>178969123</v>
+        <v>99069557</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PRA127</t>
+          <t>AFB130</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>PRA127CF</t>
+          <t>AFB130TC</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>PRA127CF</t>
+          <t>AFB130TC</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>61.13</v>
+        <v>114.1</v>
       </c>
       <c r="H47" t="n">
         <v>1</v>
       </c>
-      <c r="I47" t="n">
-        <v>1</v>
-      </c>
-      <c r="J47" t="n">
-        <v>3</v>
-      </c>
-      <c r="K47" t="n">
+      <c r="M47" t="n">
+        <v>1</v>
+      </c>
+      <c r="N47" t="n">
+        <v>2</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2</v>
+      </c>
+      <c r="P47" t="n">
         <v>4</v>
       </c>
-      <c r="L47" t="n">
-        <v>3</v>
-      </c>
-      <c r="M47" t="n">
-        <v>3</v>
-      </c>
-      <c r="N47" t="n">
+      <c r="Q47" t="n">
+        <v>2</v>
+      </c>
+      <c r="R47" t="n">
         <v>1</v>
       </c>
       <c r="U47" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="V47" t="n">
-        <v>916.95</v>
+        <v>1369.2</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>105856</v>
+        <v>105844</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2964,57 +2769,60 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>226774175</v>
+        <v>21043</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PRA728</t>
+          <t>ASF711</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>PRA728FD</t>
+          <t>ASF711CF</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>PRA728FD</t>
+          <t>ASF711CF</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>70.93000000000001</v>
+        <v>74.66</v>
       </c>
       <c r="H48" t="n">
         <v>1</v>
       </c>
-      <c r="I48" t="n">
-        <v>1</v>
-      </c>
-      <c r="J48" t="n">
-        <v>3</v>
-      </c>
-      <c r="K48" t="n">
-        <v>4</v>
-      </c>
-      <c r="L48" t="n">
-        <v>3</v>
-      </c>
       <c r="M48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N48" t="n">
+        <v>2</v>
+      </c>
+      <c r="O48" t="n">
+        <v>3</v>
+      </c>
+      <c r="P48" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>3</v>
+      </c>
+      <c r="R48" t="n">
+        <v>2</v>
+      </c>
+      <c r="S48" t="n">
         <v>1</v>
       </c>
       <c r="U48" t="n">
         <v>15</v>
       </c>
       <c r="V48" t="n">
-        <v>1063.95</v>
+        <v>1119.9</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>105856</v>
+        <v>105844</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -3022,109 +2830,989 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>226774176</v>
+        <v>62522833</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PRA728</t>
+          <t>SLB034</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>PRA728VO</t>
+          <t>SLB034PT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>PRA728VO</t>
+          <t>SLB034PT</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>70.93000000000001</v>
+        <v>200.54</v>
       </c>
       <c r="H49" t="n">
         <v>1</v>
       </c>
-      <c r="I49" t="n">
-        <v>1</v>
-      </c>
-      <c r="J49" t="n">
-        <v>2</v>
-      </c>
-      <c r="K49" t="n">
-        <v>3</v>
-      </c>
-      <c r="L49" t="n">
-        <v>3</v>
-      </c>
-      <c r="M49" t="n">
-        <v>2</v>
-      </c>
       <c r="N49" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="O49" t="n">
+        <v>3</v>
+      </c>
+      <c r="P49" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>4</v>
+      </c>
+      <c r="R49" t="n">
+        <v>3</v>
+      </c>
+      <c r="S49" t="n">
+        <v>2</v>
       </c>
       <c r="U49" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="V49" t="n">
-        <v>851.16</v>
+        <v>3609.72</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
+        <v>105844</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>164567877</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>SLB034</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SLB034TN</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>SLB034TN</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>200.54</v>
+      </c>
+      <c r="H50" t="n">
+        <v>1</v>
+      </c>
+      <c r="M50" t="n">
+        <v>1</v>
+      </c>
+      <c r="N50" t="n">
+        <v>1</v>
+      </c>
+      <c r="O50" t="n">
+        <v>4</v>
+      </c>
+      <c r="P50" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>3</v>
+      </c>
+      <c r="R50" t="n">
+        <v>1</v>
+      </c>
+      <c r="S50" t="n">
+        <v>1</v>
+      </c>
+      <c r="U50" t="n">
+        <v>15</v>
+      </c>
+      <c r="V50" t="n">
+        <v>3008.1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>105844</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>179157149</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>SWL134</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SWL134CF</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>SWL134CF</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>183.09</v>
+      </c>
+      <c r="H51" t="n">
+        <v>1</v>
+      </c>
+      <c r="M51" t="n">
+        <v>1</v>
+      </c>
+      <c r="N51" t="n">
+        <v>2</v>
+      </c>
+      <c r="O51" t="n">
+        <v>3</v>
+      </c>
+      <c r="P51" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>2</v>
+      </c>
+      <c r="R51" t="n">
+        <v>2</v>
+      </c>
+      <c r="S51" t="n">
+        <v>1</v>
+      </c>
+      <c r="U51" t="n">
+        <v>14</v>
+      </c>
+      <c r="V51" t="n">
+        <v>2563.26</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>105844</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>226799445</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>WSCR57</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>WSCR57BI</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>WSCR57BI</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>159.25</v>
+      </c>
+      <c r="H52" t="n">
+        <v>1</v>
+      </c>
+      <c r="I52" t="n">
+        <v>1</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M52" t="n">
+        <v>2</v>
+      </c>
+      <c r="N52" t="n">
+        <v>1</v>
+      </c>
+      <c r="U52" t="n">
+        <v>15</v>
+      </c>
+      <c r="V52" t="n">
+        <v>2388.75</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>105844</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>226799459</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>WSCR89</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>WSCR89TN</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>WSCR89TN</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>161.58</v>
+      </c>
+      <c r="H53" t="n">
+        <v>1</v>
+      </c>
+      <c r="I53" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" t="n">
+        <v>4</v>
+      </c>
+      <c r="L53" t="n">
+        <v>4</v>
+      </c>
+      <c r="M53" t="n">
+        <v>2</v>
+      </c>
+      <c r="N53" t="n">
+        <v>1</v>
+      </c>
+      <c r="U53" t="n">
+        <v>15</v>
+      </c>
+      <c r="V53" t="n">
+        <v>2423.7</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>105845</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>227068437</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>SAF126</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SAF126BK</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SAF126BK</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>135.3</v>
+      </c>
+      <c r="H54" t="n">
+        <v>1</v>
+      </c>
+      <c r="M54" t="n">
+        <v>1</v>
+      </c>
+      <c r="N54" t="n">
+        <v>3</v>
+      </c>
+      <c r="O54" t="n">
+        <v>4</v>
+      </c>
+      <c r="P54" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>3</v>
+      </c>
+      <c r="R54" t="n">
+        <v>2</v>
+      </c>
+      <c r="S54" t="n">
+        <v>1</v>
+      </c>
+      <c r="U54" t="n">
+        <v>18</v>
+      </c>
+      <c r="V54" t="n">
+        <v>2435.4</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>105845</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>194597523</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>SRF025</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SRF025MR</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>SRF025MR</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>153.55</v>
+      </c>
+      <c r="H55" t="n">
+        <v>1</v>
+      </c>
+      <c r="M55" t="n">
+        <v>1</v>
+      </c>
+      <c r="N55" t="n">
+        <v>3</v>
+      </c>
+      <c r="O55" t="n">
+        <v>3</v>
+      </c>
+      <c r="P55" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>2</v>
+      </c>
+      <c r="R55" t="n">
+        <v>2</v>
+      </c>
+      <c r="S55" t="n">
+        <v>1</v>
+      </c>
+      <c r="U55" t="n">
+        <v>15</v>
+      </c>
+      <c r="V55" t="n">
+        <v>2303.25</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>105845</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>226787944</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>SRT028</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SRT028BK</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>SRT028BK</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>159.78</v>
+      </c>
+      <c r="H56" t="n">
+        <v>1</v>
+      </c>
+      <c r="M56" t="n">
+        <v>1</v>
+      </c>
+      <c r="N56" t="n">
+        <v>3</v>
+      </c>
+      <c r="O56" t="n">
+        <v>4</v>
+      </c>
+      <c r="P56" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>3</v>
+      </c>
+      <c r="R56" t="n">
+        <v>2</v>
+      </c>
+      <c r="S56" t="n">
+        <v>1</v>
+      </c>
+      <c r="U56" t="n">
+        <v>18</v>
+      </c>
+      <c r="V56" t="n">
+        <v>2876.04</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>105845</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>160831013</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>SVS027</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SVS027CM</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>SVS027CM</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>145.11</v>
+      </c>
+      <c r="H57" t="n">
+        <v>1</v>
+      </c>
+      <c r="M57" t="n">
+        <v>1</v>
+      </c>
+      <c r="N57" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" t="n">
+        <v>3</v>
+      </c>
+      <c r="P57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>3</v>
+      </c>
+      <c r="U57" t="n">
+        <v>12</v>
+      </c>
+      <c r="V57" t="n">
+        <v>1741.32</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>105845</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>99645682</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>WSC003</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>WSC003OW</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>WSC003OW</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>138.2</v>
+      </c>
+      <c r="H58" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" t="n">
+        <v>1</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" t="n">
+        <v>4</v>
+      </c>
+      <c r="L58" t="n">
+        <v>5</v>
+      </c>
+      <c r="M58" t="n">
+        <v>3</v>
+      </c>
+      <c r="N58" t="n">
+        <v>1</v>
+      </c>
+      <c r="U58" t="n">
+        <v>15</v>
+      </c>
+      <c r="V58" t="n">
+        <v>2073</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>105851</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>13222</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>HCT173</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>HCT173CF</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>HCT173CF</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>52.89</v>
+      </c>
+      <c r="H59" t="n">
+        <v>1</v>
+      </c>
+      <c r="T59" t="n">
+        <v>9</v>
+      </c>
+      <c r="U59" t="n">
+        <v>9</v>
+      </c>
+      <c r="V59" t="n">
+        <v>476.01</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>105851</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>13223</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>HCT173</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>HCT173PT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>HCT173PT</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>52.89</v>
+      </c>
+      <c r="H60" t="n">
+        <v>1</v>
+      </c>
+      <c r="T60" t="n">
+        <v>6</v>
+      </c>
+      <c r="U60" t="n">
+        <v>6</v>
+      </c>
+      <c r="V60" t="n">
+        <v>317.34</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>105851</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>138654477</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>MCC008</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>MCC008TN</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>MCC008TN</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>39.04</v>
+      </c>
+      <c r="H61" t="n">
+        <v>1</v>
+      </c>
+      <c r="T61" t="n">
+        <v>9</v>
+      </c>
+      <c r="U61" t="n">
+        <v>9</v>
+      </c>
+      <c r="V61" t="n">
+        <v>351.36</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>105851</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>138654478</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>MCC008</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>MCC008VR</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>MCC008VR</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>39.04</v>
+      </c>
+      <c r="H62" t="n">
+        <v>1</v>
+      </c>
+      <c r="T62" t="n">
+        <v>9</v>
+      </c>
+      <c r="U62" t="n">
+        <v>9</v>
+      </c>
+      <c r="V62" t="n">
+        <v>351.36</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
         <v>105856</v>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>SH. NOVA AMERICA</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>178969123</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>PRA127</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>PRA127CF</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>PRA127CF</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>61.13</v>
+      </c>
+      <c r="H63" t="n">
+        <v>1</v>
+      </c>
+      <c r="I63" t="n">
+        <v>1</v>
+      </c>
+      <c r="J63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K63" t="n">
+        <v>4</v>
+      </c>
+      <c r="L63" t="n">
+        <v>3</v>
+      </c>
+      <c r="M63" t="n">
+        <v>3</v>
+      </c>
+      <c r="N63" t="n">
+        <v>1</v>
+      </c>
+      <c r="U63" t="n">
+        <v>15</v>
+      </c>
+      <c r="V63" t="n">
+        <v>916.95</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>105856</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>226774175</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>PRA728</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>PRA728FD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>PRA728FD</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="H64" t="n">
+        <v>1</v>
+      </c>
+      <c r="I64" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" t="n">
+        <v>3</v>
+      </c>
+      <c r="K64" t="n">
+        <v>4</v>
+      </c>
+      <c r="L64" t="n">
+        <v>3</v>
+      </c>
+      <c r="M64" t="n">
+        <v>3</v>
+      </c>
+      <c r="N64" t="n">
+        <v>1</v>
+      </c>
+      <c r="U64" t="n">
+        <v>15</v>
+      </c>
+      <c r="V64" t="n">
+        <v>1063.95</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>105856</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>226774176</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>PRA728</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>PRA728VO</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>PRA728VO</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="H65" t="n">
+        <v>1</v>
+      </c>
+      <c r="I65" t="n">
+        <v>1</v>
+      </c>
+      <c r="J65" t="n">
+        <v>2</v>
+      </c>
+      <c r="K65" t="n">
+        <v>3</v>
+      </c>
+      <c r="L65" t="n">
+        <v>3</v>
+      </c>
+      <c r="M65" t="n">
+        <v>2</v>
+      </c>
+      <c r="N65" t="n">
+        <v>1</v>
+      </c>
+      <c r="U65" t="n">
+        <v>12</v>
+      </c>
+      <c r="V65" t="n">
+        <v>851.16</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>105856</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SH. NOVA AMERICA</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
         <v>226799120</v>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>TBC207</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>TBC207CA</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>TBC207CA</t>
         </is>
       </c>
-      <c r="G50" t="n">
+      <c r="G66" t="n">
         <v>56.96</v>
       </c>
-      <c r="H50" t="n">
-        <v>1</v>
-      </c>
-      <c r="I50" t="n">
-        <v>1</v>
-      </c>
-      <c r="J50" t="n">
-        <v>3</v>
-      </c>
-      <c r="K50" t="n">
+      <c r="H66" t="n">
+        <v>1</v>
+      </c>
+      <c r="I66" t="n">
+        <v>1</v>
+      </c>
+      <c r="J66" t="n">
+        <v>3</v>
+      </c>
+      <c r="K66" t="n">
         <v>5</v>
       </c>
-      <c r="L50" t="n">
+      <c r="L66" t="n">
         <v>4</v>
       </c>
-      <c r="M50" t="n">
-        <v>3</v>
-      </c>
-      <c r="N50" t="n">
-        <v>2</v>
-      </c>
-      <c r="U50" t="n">
+      <c r="M66" t="n">
+        <v>3</v>
+      </c>
+      <c r="N66" t="n">
+        <v>2</v>
+      </c>
+      <c r="U66" t="n">
         <v>18</v>
       </c>
-      <c r="V50" t="n">
+      <c r="V66" t="n">
         <v>1025.28</v>
       </c>
     </row>
@@ -3351,15 +4039,26 @@
           <t>CLASSE COURO DISTRIBUIDORA</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>N3_RelB2bCarrinhoExcel-18h47.xlsx</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEM ARQUIVO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>65</v>
       </c>
+      <c r="G6" t="n">
+        <v>65</v>
+      </c>
       <c r="H6" t="n">
+        <v>6516.57</v>
+      </c>
+      <c r="I6" t="n">
         <v>6516.57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add departamento, categoria and colecao to unified spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Nova_America_Unificado.xlsx
+++ b/pedidos/Pedidos_Nova_America_Unificado.xlsx
@@ -30,12 +30,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -50,9 +55,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V66"/>
+  <dimension ref="A1:Y66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,58 +460,73 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Coleção</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Preço</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Qtd Caixas</t>
         </is>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="L1" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="M1" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="N1" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="O1" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="P1" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="Q1" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="R1" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="S1" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="T1" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="U1" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="V1" s="1" t="n">
         <v>44</v>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>UN</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Qtd Total</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Vlr Total</t>
         </is>
@@ -528,47 +549,50 @@
           <t>CAR112</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>CAR112PT</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>CAR112PT</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" t="n">
         <v>268.14</v>
       </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O2" t="n">
-        <v>3</v>
+      <c r="K2" t="n">
+        <v>1</v>
       </c>
       <c r="P2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S2" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="T2" t="n">
+        <v>3</v>
       </c>
       <c r="U2" t="n">
+        <v>2</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" t="n">
         <v>15</v>
       </c>
-      <c r="V2" t="n">
+      <c r="Y2" t="n">
         <v>4022.1</v>
       </c>
     </row>
@@ -599,37 +623,52 @@
           <t>DSG125PH</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>SOCIAL</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>VERAO</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
         <v>209.1</v>
       </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1</v>
-      </c>
-      <c r="N3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O3" t="n">
-        <v>3</v>
+      <c r="K3" t="n">
+        <v>1</v>
       </c>
       <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>2</v>
+      </c>
+      <c r="R3" t="n">
+        <v>3</v>
+      </c>
+      <c r="S3" t="n">
         <v>4</v>
       </c>
-      <c r="Q3" t="n">
-        <v>3</v>
-      </c>
-      <c r="R3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S3" t="n">
-        <v>1</v>
+      <c r="T3" t="n">
+        <v>3</v>
       </c>
       <c r="U3" t="n">
+        <v>1</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
         <v>15</v>
       </c>
-      <c r="V3" t="n">
+      <c r="Y3" t="n">
         <v>3136.5</v>
       </c>
     </row>
@@ -650,47 +689,50 @@
           <t>SLG010</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>SLG010PT</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>SLG010PT</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" t="n">
         <v>242.31</v>
       </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O4" t="n">
-        <v>3</v>
+      <c r="K4" t="n">
+        <v>1</v>
       </c>
       <c r="P4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S4" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="T4" t="n">
+        <v>3</v>
       </c>
       <c r="U4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
         <v>15</v>
       </c>
-      <c r="V4" t="n">
+      <c r="Y4" t="n">
         <v>3634.65</v>
       </c>
     </row>
@@ -721,22 +763,37 @@
           <t>LMM016BG</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
         <v>19.91</v>
       </c>
-      <c r="H5" t="n">
-        <v>1</v>
-      </c>
       <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
         <v>12</v>
       </c>
-      <c r="O5" t="n">
+      <c r="R5" t="n">
         <v>12</v>
       </c>
-      <c r="U5" t="n">
+      <c r="X5" t="n">
         <v>24</v>
       </c>
-      <c r="V5" t="n">
+      <c r="Y5" t="n">
         <v>477.84</v>
       </c>
     </row>
@@ -767,22 +824,37 @@
           <t>LMM016PT</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
         <v>19.91</v>
       </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
       <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
         <v>24</v>
       </c>
-      <c r="O6" t="n">
+      <c r="R6" t="n">
         <v>24</v>
       </c>
-      <c r="U6" t="n">
+      <c r="X6" t="n">
         <v>48</v>
       </c>
-      <c r="V6" t="n">
+      <c r="Y6" t="n">
         <v>955.6799999999999</v>
       </c>
     </row>
@@ -803,44 +875,47 @@
           <t>PRA747</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>PRA747CF</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>PRA747CF</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" t="n">
         <v>54.9</v>
       </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="n">
-        <v>2</v>
-      </c>
       <c r="K7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
         <v>2</v>
       </c>
       <c r="N7" t="n">
-        <v>1</v>
-      </c>
-      <c r="U7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
         <v>12</v>
       </c>
-      <c r="V7" t="n">
+      <c r="Y7" t="n">
         <v>658.8</v>
       </c>
     </row>
@@ -861,44 +936,47 @@
           <t>TBE004</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>TBE004BI</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>TBE004BI</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" t="n">
         <v>60.88</v>
       </c>
-      <c r="H8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="n">
-        <v>3</v>
-      </c>
       <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="n">
         <v>4</v>
       </c>
-      <c r="L8" t="n">
+      <c r="O8" t="n">
         <v>4</v>
       </c>
-      <c r="M8" t="n">
-        <v>2</v>
-      </c>
-      <c r="N8" t="n">
-        <v>1</v>
-      </c>
-      <c r="U8" t="n">
+      <c r="P8" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
         <v>15</v>
       </c>
-      <c r="V8" t="n">
+      <c r="Y8" t="n">
         <v>913.2</v>
       </c>
     </row>
@@ -919,44 +997,47 @@
           <t>TBE004</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>TBE004OU</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>TBE004OU</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" t="n">
         <v>60.88</v>
       </c>
-      <c r="H9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" t="n">
-        <v>3</v>
-      </c>
       <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" t="n">
         <v>4</v>
       </c>
-      <c r="L9" t="n">
+      <c r="O9" t="n">
         <v>4</v>
       </c>
-      <c r="M9" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
-      <c r="U9" t="n">
+      <c r="P9" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
         <v>15</v>
       </c>
-      <c r="V9" t="n">
+      <c r="Y9" t="n">
         <v>913.2</v>
       </c>
     </row>
@@ -977,44 +1058,47 @@
           <t>TBE004</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>TBE004PT</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>TBE004PT</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" t="n">
         <v>60.88</v>
       </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" t="n">
-        <v>3</v>
-      </c>
       <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" t="n">
         <v>4</v>
       </c>
-      <c r="L10" t="n">
+      <c r="O10" t="n">
         <v>4</v>
       </c>
-      <c r="M10" t="n">
-        <v>2</v>
-      </c>
-      <c r="N10" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" t="n">
+      <c r="P10" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
         <v>15</v>
       </c>
-      <c r="V10" t="n">
+      <c r="Y10" t="n">
         <v>913.2</v>
       </c>
     </row>
@@ -1035,44 +1119,47 @@
           <t>TBE004</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>TBE004TN</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>TBE004TN</t>
         </is>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" t="n">
         <v>60.88</v>
       </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" t="n">
-        <v>3</v>
-      </c>
       <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N11" t="n">
         <v>4</v>
       </c>
-      <c r="L11" t="n">
+      <c r="O11" t="n">
         <v>4</v>
       </c>
-      <c r="M11" t="n">
-        <v>2</v>
-      </c>
-      <c r="N11" t="n">
-        <v>1</v>
-      </c>
-      <c r="U11" t="n">
+      <c r="P11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
         <v>15</v>
       </c>
-      <c r="V11" t="n">
+      <c r="Y11" t="n">
         <v>913.2</v>
       </c>
     </row>
@@ -1103,19 +1190,34 @@
           <t>GBF065OW</t>
         </is>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
         <v>230.4</v>
       </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" t="n">
-        <v>2</v>
-      </c>
-      <c r="U12" t="n">
-        <v>2</v>
-      </c>
-      <c r="V12" t="n">
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" t="n">
+        <v>2</v>
+      </c>
+      <c r="X12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y12" t="n">
         <v>460.8</v>
       </c>
     </row>
@@ -1146,19 +1248,34 @@
           <t>GBF801CF</t>
         </is>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
         <v>234</v>
       </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" t="n">
-        <v>3</v>
-      </c>
-      <c r="U13" t="n">
-        <v>3</v>
-      </c>
-      <c r="V13" t="n">
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="W13" t="n">
+        <v>3</v>
+      </c>
+      <c r="X13" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y13" t="n">
         <v>702</v>
       </c>
     </row>
@@ -1189,19 +1306,34 @@
           <t>GMO404CF</t>
         </is>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
         <v>240</v>
       </c>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
-      <c r="T14" t="n">
-        <v>1</v>
-      </c>
-      <c r="U14" t="n">
-        <v>1</v>
-      </c>
-      <c r="V14" t="n">
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="W14" t="n">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y14" t="n">
         <v>240</v>
       </c>
     </row>
@@ -1232,19 +1364,34 @@
           <t>GMO404PT</t>
         </is>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
         <v>240</v>
       </c>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
-      <c r="T15" t="n">
-        <v>1</v>
-      </c>
-      <c r="U15" t="n">
-        <v>1</v>
-      </c>
-      <c r="V15" t="n">
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="W15" t="n">
+        <v>1</v>
+      </c>
+      <c r="X15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" t="n">
         <v>240</v>
       </c>
     </row>
@@ -1265,44 +1412,47 @@
           <t>PAB078</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>PAB078VO</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>PAB078VO</t>
         </is>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" t="n">
         <v>149.31</v>
       </c>
-      <c r="H16" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" t="n">
-        <v>2</v>
-      </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M16" t="n">
         <v>2</v>
       </c>
       <c r="N16" t="n">
-        <v>1</v>
-      </c>
-      <c r="U16" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" t="n">
+        <v>3</v>
+      </c>
+      <c r="P16" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
         <v>12</v>
       </c>
-      <c r="V16" t="n">
+      <c r="Y16" t="n">
         <v>1791.72</v>
       </c>
     </row>
@@ -1323,44 +1473,47 @@
           <t>WCL203</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>WCL203CF</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>WCL203CF</t>
         </is>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" t="n">
         <v>145.33</v>
       </c>
-      <c r="H17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" t="n">
-        <v>2</v>
-      </c>
       <c r="K17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M17" t="n">
         <v>2</v>
       </c>
       <c r="N17" t="n">
-        <v>1</v>
-      </c>
-      <c r="U17" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" t="n">
+        <v>3</v>
+      </c>
+      <c r="P17" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
         <v>12</v>
       </c>
-      <c r="V17" t="n">
+      <c r="Y17" t="n">
         <v>1743.96</v>
       </c>
     </row>
@@ -1381,44 +1534,47 @@
           <t>WCL204</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>WCL204CA</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>WCL204CA</t>
         </is>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" t="n">
         <v>154.12</v>
       </c>
-      <c r="H18" t="n">
-        <v>1</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" t="n">
-        <v>2</v>
-      </c>
       <c r="K18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M18" t="n">
         <v>2</v>
       </c>
       <c r="N18" t="n">
-        <v>1</v>
-      </c>
-      <c r="U18" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" t="n">
+        <v>3</v>
+      </c>
+      <c r="P18" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
+      <c r="X18" t="n">
         <v>12</v>
       </c>
-      <c r="V18" t="n">
+      <c r="Y18" t="n">
         <v>1849.44</v>
       </c>
     </row>
@@ -1439,44 +1595,47 @@
           <t>WSC330</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>WSC330OU</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" t="n">
         <v>68.31999999999999</v>
       </c>
-      <c r="H19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" t="n">
-        <v>3</v>
-      </c>
       <c r="K19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" t="n">
         <v>4</v>
       </c>
-      <c r="L19" t="n">
+      <c r="O19" t="n">
         <v>5</v>
       </c>
-      <c r="M19" t="n">
-        <v>3</v>
-      </c>
-      <c r="N19" t="n">
-        <v>2</v>
-      </c>
-      <c r="U19" t="n">
+      <c r="P19" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>2</v>
+      </c>
+      <c r="X19" t="n">
         <v>18</v>
       </c>
-      <c r="V19" t="n">
+      <c r="Y19" t="n">
         <v>1229.76</v>
       </c>
     </row>
@@ -1507,34 +1666,49 @@
           <t>WSCR61PT</t>
         </is>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
         <v>118.83</v>
       </c>
-      <c r="H20" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" t="n">
-        <v>3</v>
-      </c>
       <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" t="n">
         <v>4</v>
       </c>
-      <c r="L20" t="n">
+      <c r="O20" t="n">
         <v>6</v>
       </c>
-      <c r="M20" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" t="n">
-        <v>2</v>
-      </c>
-      <c r="U20" t="n">
+      <c r="P20" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>2</v>
+      </c>
+      <c r="X20" t="n">
         <v>18</v>
       </c>
-      <c r="V20" t="n">
+      <c r="Y20" t="n">
         <v>2138.94</v>
       </c>
     </row>
@@ -1565,34 +1739,49 @@
           <t>PMD057FD</t>
         </is>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>SANDALIA SALTO</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>VERAO</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
         <v>109.2</v>
       </c>
-      <c r="H21" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" t="n">
-        <v>3</v>
-      </c>
       <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" t="n">
+        <v>3</v>
+      </c>
+      <c r="N21" t="n">
         <v>4</v>
       </c>
-      <c r="L21" t="n">
+      <c r="O21" t="n">
         <v>4</v>
       </c>
-      <c r="M21" t="n">
-        <v>2</v>
-      </c>
-      <c r="N21" t="n">
-        <v>1</v>
-      </c>
-      <c r="U21" t="n">
+      <c r="P21" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
+      <c r="X21" t="n">
         <v>15</v>
       </c>
-      <c r="V21" t="n">
+      <c r="Y21" t="n">
         <v>1638</v>
       </c>
     </row>
@@ -1613,44 +1802,47 @@
           <t>PMD407</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>PMD407CF</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>PMD407CF</t>
         </is>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" t="n">
         <v>110.18</v>
       </c>
-      <c r="H22" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" t="n">
-        <v>3</v>
-      </c>
       <c r="K22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" t="n">
         <v>4</v>
       </c>
-      <c r="L22" t="n">
+      <c r="O22" t="n">
         <v>4</v>
       </c>
-      <c r="M22" t="n">
-        <v>2</v>
-      </c>
-      <c r="N22" t="n">
-        <v>1</v>
-      </c>
-      <c r="U22" t="n">
+      <c r="P22" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1</v>
+      </c>
+      <c r="X22" t="n">
         <v>15</v>
       </c>
-      <c r="V22" t="n">
+      <c r="Y22" t="n">
         <v>1652.7</v>
       </c>
     </row>
@@ -1671,44 +1863,47 @@
           <t>PRA732</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>PRA732CF</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>PRA732CF</t>
         </is>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" t="n">
         <v>61.35</v>
       </c>
-      <c r="H23" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" t="n">
-        <v>1</v>
-      </c>
-      <c r="J23" t="n">
-        <v>3</v>
-      </c>
       <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" t="n">
         <v>4</v>
       </c>
-      <c r="L23" t="n">
-        <v>3</v>
-      </c>
-      <c r="M23" t="n">
-        <v>3</v>
-      </c>
-      <c r="N23" t="n">
-        <v>1</v>
-      </c>
-      <c r="U23" t="n">
+      <c r="O23" t="n">
+        <v>3</v>
+      </c>
+      <c r="P23" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>1</v>
+      </c>
+      <c r="X23" t="n">
         <v>15</v>
       </c>
-      <c r="V23" t="n">
+      <c r="Y23" t="n">
         <v>920.25</v>
       </c>
     </row>
@@ -1739,19 +1934,34 @@
           <t>LMM004BG</t>
         </is>
       </c>
-      <c r="G24" t="n">
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
         <v>17.51</v>
       </c>
-      <c r="H24" t="n">
-        <v>1</v>
-      </c>
-      <c r="T24" t="n">
+      <c r="K24" t="n">
+        <v>1</v>
+      </c>
+      <c r="W24" t="n">
         <v>24</v>
       </c>
-      <c r="U24" t="n">
+      <c r="X24" t="n">
         <v>24</v>
       </c>
-      <c r="V24" t="n">
+      <c r="Y24" t="n">
         <v>420.24</v>
       </c>
     </row>
@@ -1782,19 +1992,34 @@
           <t>LMM004MM</t>
         </is>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
         <v>17.51</v>
       </c>
-      <c r="H25" t="n">
-        <v>1</v>
-      </c>
-      <c r="T25" t="n">
+      <c r="K25" t="n">
+        <v>1</v>
+      </c>
+      <c r="W25" t="n">
         <v>24</v>
       </c>
-      <c r="U25" t="n">
+      <c r="X25" t="n">
         <v>24</v>
       </c>
-      <c r="V25" t="n">
+      <c r="Y25" t="n">
         <v>420.24</v>
       </c>
     </row>
@@ -1825,19 +2050,34 @@
           <t>LMM004PT</t>
         </is>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
         <v>17.51</v>
       </c>
-      <c r="H26" t="n">
-        <v>1</v>
-      </c>
-      <c r="T26" t="n">
+      <c r="K26" t="n">
+        <v>1</v>
+      </c>
+      <c r="W26" t="n">
         <v>36</v>
       </c>
-      <c r="U26" t="n">
+      <c r="X26" t="n">
         <v>36</v>
       </c>
-      <c r="V26" t="n">
+      <c r="Y26" t="n">
         <v>630.36</v>
       </c>
     </row>
@@ -1868,19 +2108,34 @@
           <t>LMM009PT</t>
         </is>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
         <v>15.63</v>
       </c>
-      <c r="H27" t="n">
-        <v>1</v>
-      </c>
-      <c r="T27" t="n">
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
+      <c r="W27" t="n">
         <v>36</v>
       </c>
-      <c r="U27" t="n">
+      <c r="X27" t="n">
         <v>36</v>
       </c>
-      <c r="V27" t="n">
+      <c r="Y27" t="n">
         <v>562.6799999999999</v>
       </c>
     </row>
@@ -1911,19 +2166,34 @@
           <t>LMM619BC</t>
         </is>
       </c>
-      <c r="G28" t="n">
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
         <v>15.33</v>
       </c>
-      <c r="H28" t="n">
-        <v>1</v>
-      </c>
-      <c r="T28" t="n">
+      <c r="K28" t="n">
+        <v>1</v>
+      </c>
+      <c r="W28" t="n">
         <v>60</v>
       </c>
-      <c r="U28" t="n">
+      <c r="X28" t="n">
         <v>60</v>
       </c>
-      <c r="V28" t="n">
+      <c r="Y28" t="n">
         <v>919.8</v>
       </c>
     </row>
@@ -1954,19 +2224,34 @@
           <t>LMM619BG</t>
         </is>
       </c>
-      <c r="G29" t="n">
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
         <v>15.33</v>
       </c>
-      <c r="H29" t="n">
-        <v>1</v>
-      </c>
-      <c r="T29" t="n">
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+      <c r="W29" t="n">
         <v>36</v>
       </c>
-      <c r="U29" t="n">
+      <c r="X29" t="n">
         <v>36</v>
       </c>
-      <c r="V29" t="n">
+      <c r="Y29" t="n">
         <v>551.88</v>
       </c>
     </row>
@@ -1997,19 +2282,34 @@
           <t>LMM619PT</t>
         </is>
       </c>
-      <c r="G30" t="n">
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>VESTUARIO</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>MEIAS</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
         <v>15.33</v>
       </c>
-      <c r="H30" t="n">
-        <v>1</v>
-      </c>
-      <c r="T30" t="n">
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="W30" t="n">
         <v>60</v>
       </c>
-      <c r="U30" t="n">
+      <c r="X30" t="n">
         <v>60</v>
       </c>
-      <c r="V30" t="n">
+      <c r="Y30" t="n">
         <v>919.8</v>
       </c>
     </row>
@@ -2030,29 +2330,32 @@
           <t>GBF191</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>GBF191CF</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>GBF191CF</t>
         </is>
       </c>
-      <c r="G31" t="n">
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" t="n">
         <v>242.99</v>
       </c>
-      <c r="H31" t="n">
-        <v>1</v>
-      </c>
-      <c r="T31" t="n">
-        <v>2</v>
-      </c>
-      <c r="U31" t="n">
-        <v>2</v>
-      </c>
-      <c r="V31" t="n">
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
+      <c r="W31" t="n">
+        <v>2</v>
+      </c>
+      <c r="X31" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y31" t="n">
         <v>485.98</v>
       </c>
     </row>
@@ -2073,29 +2376,32 @@
           <t>GBF191</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>GBF191VO</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>GBF191VO</t>
         </is>
       </c>
-      <c r="G32" t="n">
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" t="n">
         <v>242.99</v>
       </c>
-      <c r="H32" t="n">
-        <v>1</v>
-      </c>
-      <c r="T32" t="n">
-        <v>2</v>
-      </c>
-      <c r="U32" t="n">
-        <v>2</v>
-      </c>
-      <c r="V32" t="n">
+      <c r="K32" t="n">
+        <v>1</v>
+      </c>
+      <c r="W32" t="n">
+        <v>2</v>
+      </c>
+      <c r="X32" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y32" t="n">
         <v>485.98</v>
       </c>
     </row>
@@ -2116,29 +2422,32 @@
           <t>GBF269</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>GBF269FD</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>GBF269FD</t>
         </is>
       </c>
-      <c r="G33" t="n">
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" t="n">
         <v>235</v>
       </c>
-      <c r="H33" t="n">
-        <v>1</v>
-      </c>
-      <c r="T33" t="n">
-        <v>2</v>
-      </c>
-      <c r="U33" t="n">
-        <v>2</v>
-      </c>
-      <c r="V33" t="n">
+      <c r="K33" t="n">
+        <v>1</v>
+      </c>
+      <c r="W33" t="n">
+        <v>2</v>
+      </c>
+      <c r="X33" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y33" t="n">
         <v>470</v>
       </c>
     </row>
@@ -2169,19 +2478,34 @@
           <t>GBF445CF</t>
         </is>
       </c>
-      <c r="G34" t="n">
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>VERAO</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
         <v>122.67</v>
       </c>
-      <c r="H34" t="n">
-        <v>1</v>
-      </c>
-      <c r="T34" t="n">
-        <v>2</v>
-      </c>
-      <c r="U34" t="n">
-        <v>2</v>
-      </c>
-      <c r="V34" t="n">
+      <c r="K34" t="n">
+        <v>1</v>
+      </c>
+      <c r="W34" t="n">
+        <v>2</v>
+      </c>
+      <c r="X34" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y34" t="n">
         <v>245.34</v>
       </c>
     </row>
@@ -2212,19 +2536,34 @@
           <t>GBF445PT</t>
         </is>
       </c>
-      <c r="G35" t="n">
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
         <v>122.67</v>
       </c>
-      <c r="H35" t="n">
-        <v>1</v>
-      </c>
-      <c r="T35" t="n">
-        <v>3</v>
-      </c>
-      <c r="U35" t="n">
-        <v>3</v>
-      </c>
-      <c r="V35" t="n">
+      <c r="K35" t="n">
+        <v>1</v>
+      </c>
+      <c r="W35" t="n">
+        <v>3</v>
+      </c>
+      <c r="X35" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y35" t="n">
         <v>368.01</v>
       </c>
     </row>
@@ -2245,29 +2584,32 @@
           <t>GBF786</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>GBF786CF</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>GBF786CF</t>
         </is>
       </c>
-      <c r="G36" t="n">
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" t="n">
         <v>200.69</v>
       </c>
-      <c r="H36" t="n">
-        <v>1</v>
-      </c>
-      <c r="T36" t="n">
-        <v>2</v>
-      </c>
-      <c r="U36" t="n">
-        <v>2</v>
-      </c>
-      <c r="V36" t="n">
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="W36" t="n">
+        <v>2</v>
+      </c>
+      <c r="X36" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y36" t="n">
         <v>401.38</v>
       </c>
     </row>
@@ -2288,29 +2630,32 @@
           <t>GBF788</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>GBF788PT</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>GBF788PT</t>
         </is>
       </c>
-      <c r="G37" t="n">
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" t="n">
         <v>138.06</v>
       </c>
-      <c r="H37" t="n">
-        <v>1</v>
-      </c>
-      <c r="T37" t="n">
-        <v>3</v>
-      </c>
-      <c r="U37" t="n">
-        <v>3</v>
-      </c>
-      <c r="V37" t="n">
+      <c r="K37" t="n">
+        <v>1</v>
+      </c>
+      <c r="W37" t="n">
+        <v>3</v>
+      </c>
+      <c r="X37" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y37" t="n">
         <v>414.18</v>
       </c>
     </row>
@@ -2331,29 +2676,32 @@
           <t>GBF788</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>GBF788TN</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>GBF788TN</t>
         </is>
       </c>
-      <c r="G38" t="n">
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" t="n">
         <v>138.06</v>
       </c>
-      <c r="H38" t="n">
-        <v>1</v>
-      </c>
-      <c r="T38" t="n">
-        <v>3</v>
-      </c>
-      <c r="U38" t="n">
-        <v>3</v>
-      </c>
-      <c r="V38" t="n">
+      <c r="K38" t="n">
+        <v>1</v>
+      </c>
+      <c r="W38" t="n">
+        <v>3</v>
+      </c>
+      <c r="X38" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y38" t="n">
         <v>414.18</v>
       </c>
     </row>
@@ -2384,19 +2732,34 @@
           <t>GBF827PT</t>
         </is>
       </c>
-      <c r="G39" t="n">
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
         <v>85.78</v>
       </c>
-      <c r="H39" t="n">
-        <v>1</v>
-      </c>
-      <c r="T39" t="n">
+      <c r="K39" t="n">
+        <v>1</v>
+      </c>
+      <c r="W39" t="n">
         <v>8</v>
       </c>
-      <c r="U39" t="n">
+      <c r="X39" t="n">
         <v>8</v>
       </c>
-      <c r="V39" t="n">
+      <c r="Y39" t="n">
         <v>686.24</v>
       </c>
     </row>
@@ -2427,19 +2790,34 @@
           <t>GSN810PT</t>
         </is>
       </c>
-      <c r="G40" t="n">
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
         <v>122.2</v>
       </c>
-      <c r="H40" t="n">
-        <v>1</v>
-      </c>
-      <c r="T40" t="n">
-        <v>2</v>
-      </c>
-      <c r="U40" t="n">
-        <v>2</v>
-      </c>
-      <c r="V40" t="n">
+      <c r="K40" t="n">
+        <v>1</v>
+      </c>
+      <c r="W40" t="n">
+        <v>2</v>
+      </c>
+      <c r="X40" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y40" t="n">
         <v>244.4</v>
       </c>
     </row>
@@ -2470,19 +2848,34 @@
           <t>GSN811PT</t>
         </is>
       </c>
-      <c r="G41" t="n">
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
         <v>123.38</v>
       </c>
-      <c r="H41" t="n">
-        <v>1</v>
-      </c>
-      <c r="T41" t="n">
+      <c r="K41" t="n">
+        <v>1</v>
+      </c>
+      <c r="W41" t="n">
         <v>4</v>
       </c>
-      <c r="U41" t="n">
+      <c r="X41" t="n">
         <v>4</v>
       </c>
-      <c r="V41" t="n">
+      <c r="Y41" t="n">
         <v>493.52</v>
       </c>
     </row>
@@ -2513,19 +2906,34 @@
           <t>GSN811TN</t>
         </is>
       </c>
-      <c r="G42" t="n">
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>BOLSA</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
         <v>123.38</v>
       </c>
-      <c r="H42" t="n">
-        <v>1</v>
-      </c>
-      <c r="T42" t="n">
+      <c r="K42" t="n">
+        <v>1</v>
+      </c>
+      <c r="W42" t="n">
         <v>4</v>
       </c>
-      <c r="U42" t="n">
+      <c r="X42" t="n">
         <v>4</v>
       </c>
-      <c r="V42" t="n">
+      <c r="Y42" t="n">
         <v>493.52</v>
       </c>
     </row>
@@ -2556,19 +2964,34 @@
           <t>HCT054CF</t>
         </is>
       </c>
-      <c r="G43" t="n">
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>CARTEIRA</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
         <v>45.77</v>
       </c>
-      <c r="H43" t="n">
-        <v>1</v>
-      </c>
-      <c r="T43" t="n">
+      <c r="K43" t="n">
+        <v>1</v>
+      </c>
+      <c r="W43" t="n">
         <v>4</v>
       </c>
-      <c r="U43" t="n">
+      <c r="X43" t="n">
         <v>4</v>
       </c>
-      <c r="V43" t="n">
+      <c r="Y43" t="n">
         <v>183.08</v>
       </c>
     </row>
@@ -2599,19 +3022,34 @@
           <t>HCT054PT</t>
         </is>
       </c>
-      <c r="G44" t="n">
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>CARTEIRA</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
         <v>45.77</v>
       </c>
-      <c r="H44" t="n">
-        <v>1</v>
-      </c>
-      <c r="T44" t="n">
+      <c r="K44" t="n">
+        <v>1</v>
+      </c>
+      <c r="W44" t="n">
         <v>9</v>
       </c>
-      <c r="U44" t="n">
+      <c r="X44" t="n">
         <v>9</v>
       </c>
-      <c r="V44" t="n">
+      <c r="Y44" t="n">
         <v>411.93</v>
       </c>
     </row>
@@ -2642,19 +3080,34 @@
           <t>HCT095PT</t>
         </is>
       </c>
-      <c r="G45" t="n">
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>CARTEIRA</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
         <v>49.35</v>
       </c>
-      <c r="H45" t="n">
-        <v>1</v>
-      </c>
-      <c r="T45" t="n">
+      <c r="K45" t="n">
+        <v>1</v>
+      </c>
+      <c r="W45" t="n">
         <v>9</v>
       </c>
-      <c r="U45" t="n">
+      <c r="X45" t="n">
         <v>9</v>
       </c>
-      <c r="V45" t="n">
+      <c r="Y45" t="n">
         <v>444.15</v>
       </c>
     </row>
@@ -2685,19 +3138,34 @@
           <t>HCT096PT</t>
         </is>
       </c>
-      <c r="G46" t="n">
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>CARTEIRA</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
         <v>45.78</v>
       </c>
-      <c r="H46" t="n">
-        <v>1</v>
-      </c>
-      <c r="T46" t="n">
+      <c r="K46" t="n">
+        <v>1</v>
+      </c>
+      <c r="W46" t="n">
         <v>6</v>
       </c>
-      <c r="U46" t="n">
+      <c r="X46" t="n">
         <v>6</v>
       </c>
-      <c r="V46" t="n">
+      <c r="Y46" t="n">
         <v>274.68</v>
       </c>
     </row>
@@ -2728,34 +3196,49 @@
           <t>AFB130TC</t>
         </is>
       </c>
-      <c r="G47" t="n">
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>MOCASSIM</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
         <v>114.1</v>
       </c>
-      <c r="H47" t="n">
-        <v>1</v>
-      </c>
-      <c r="M47" t="n">
-        <v>1</v>
-      </c>
-      <c r="N47" t="n">
-        <v>2</v>
-      </c>
-      <c r="O47" t="n">
-        <v>2</v>
+      <c r="K47" t="n">
+        <v>1</v>
       </c>
       <c r="P47" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2</v>
+      </c>
+      <c r="R47" t="n">
+        <v>2</v>
+      </c>
+      <c r="S47" t="n">
         <v>4</v>
       </c>
-      <c r="Q47" t="n">
-        <v>2</v>
-      </c>
-      <c r="R47" t="n">
-        <v>1</v>
+      <c r="T47" t="n">
+        <v>2</v>
       </c>
       <c r="U47" t="n">
+        <v>1</v>
+      </c>
+      <c r="X47" t="n">
         <v>12</v>
       </c>
-      <c r="V47" t="n">
+      <c r="Y47" t="n">
         <v>1369.2</v>
       </c>
     </row>
@@ -2786,37 +3269,52 @@
           <t>ASF711CF</t>
         </is>
       </c>
-      <c r="G48" t="n">
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>SANDALIA</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
         <v>74.66</v>
       </c>
-      <c r="H48" t="n">
-        <v>1</v>
-      </c>
-      <c r="M48" t="n">
-        <v>1</v>
-      </c>
-      <c r="N48" t="n">
-        <v>2</v>
-      </c>
-      <c r="O48" t="n">
-        <v>3</v>
+      <c r="K48" t="n">
+        <v>1</v>
       </c>
       <c r="P48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S48" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="T48" t="n">
+        <v>3</v>
       </c>
       <c r="U48" t="n">
+        <v>2</v>
+      </c>
+      <c r="V48" t="n">
+        <v>1</v>
+      </c>
+      <c r="X48" t="n">
         <v>15</v>
       </c>
-      <c r="V48" t="n">
+      <c r="Y48" t="n">
         <v>1119.9</v>
       </c>
     </row>
@@ -2847,34 +3345,49 @@
           <t>SLB034PT</t>
         </is>
       </c>
-      <c r="G49" t="n">
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
         <v>200.54</v>
       </c>
-      <c r="H49" t="n">
-        <v>1</v>
-      </c>
-      <c r="N49" t="n">
-        <v>2</v>
-      </c>
-      <c r="O49" t="n">
-        <v>3</v>
-      </c>
-      <c r="P49" t="n">
+      <c r="K49" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2</v>
+      </c>
+      <c r="R49" t="n">
+        <v>3</v>
+      </c>
+      <c r="S49" t="n">
         <v>4</v>
       </c>
-      <c r="Q49" t="n">
+      <c r="T49" t="n">
         <v>4</v>
       </c>
-      <c r="R49" t="n">
-        <v>3</v>
-      </c>
-      <c r="S49" t="n">
-        <v>2</v>
-      </c>
       <c r="U49" t="n">
+        <v>3</v>
+      </c>
+      <c r="V49" t="n">
+        <v>2</v>
+      </c>
+      <c r="X49" t="n">
         <v>18</v>
       </c>
-      <c r="V49" t="n">
+      <c r="Y49" t="n">
         <v>3609.72</v>
       </c>
     </row>
@@ -2905,37 +3418,52 @@
           <t>SLB034TN</t>
         </is>
       </c>
-      <c r="G50" t="n">
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
         <v>200.54</v>
       </c>
-      <c r="H50" t="n">
-        <v>1</v>
-      </c>
-      <c r="M50" t="n">
-        <v>1</v>
-      </c>
-      <c r="N50" t="n">
-        <v>1</v>
-      </c>
-      <c r="O50" t="n">
+      <c r="K50" t="n">
+        <v>1</v>
+      </c>
+      <c r="P50" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>1</v>
+      </c>
+      <c r="R50" t="n">
         <v>4</v>
       </c>
-      <c r="P50" t="n">
+      <c r="S50" t="n">
         <v>4</v>
       </c>
-      <c r="Q50" t="n">
-        <v>3</v>
-      </c>
-      <c r="R50" t="n">
-        <v>1</v>
-      </c>
-      <c r="S50" t="n">
-        <v>1</v>
+      <c r="T50" t="n">
+        <v>3</v>
       </c>
       <c r="U50" t="n">
+        <v>1</v>
+      </c>
+      <c r="V50" t="n">
+        <v>1</v>
+      </c>
+      <c r="X50" t="n">
         <v>15</v>
       </c>
-      <c r="V50" t="n">
+      <c r="Y50" t="n">
         <v>3008.1</v>
       </c>
     </row>
@@ -2966,37 +3494,52 @@
           <t>SWL134CF</t>
         </is>
       </c>
-      <c r="G51" t="n">
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
         <v>183.09</v>
       </c>
-      <c r="H51" t="n">
-        <v>1</v>
-      </c>
-      <c r="M51" t="n">
-        <v>1</v>
-      </c>
-      <c r="N51" t="n">
-        <v>2</v>
-      </c>
-      <c r="O51" t="n">
-        <v>3</v>
+      <c r="K51" t="n">
+        <v>1</v>
       </c>
       <c r="P51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q51" t="n">
         <v>2</v>
       </c>
       <c r="R51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S51" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="T51" t="n">
+        <v>2</v>
       </c>
       <c r="U51" t="n">
+        <v>2</v>
+      </c>
+      <c r="V51" t="n">
+        <v>1</v>
+      </c>
+      <c r="X51" t="n">
         <v>14</v>
       </c>
-      <c r="V51" t="n">
+      <c r="Y51" t="n">
         <v>2563.26</v>
       </c>
     </row>
@@ -3017,44 +3560,47 @@
           <t>WSCR57</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>WSCR57BI</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>WSCR57BI</t>
         </is>
       </c>
-      <c r="G52" t="n">
+      <c r="G52" s="2" t="n"/>
+      <c r="H52" s="2" t="n"/>
+      <c r="I52" s="2" t="n"/>
+      <c r="J52" t="n">
         <v>159.25</v>
       </c>
-      <c r="H52" t="n">
-        <v>1</v>
-      </c>
-      <c r="I52" t="n">
-        <v>1</v>
-      </c>
-      <c r="J52" t="n">
-        <v>3</v>
-      </c>
       <c r="K52" t="n">
+        <v>1</v>
+      </c>
+      <c r="L52" t="n">
+        <v>1</v>
+      </c>
+      <c r="M52" t="n">
+        <v>3</v>
+      </c>
+      <c r="N52" t="n">
         <v>4</v>
       </c>
-      <c r="L52" t="n">
+      <c r="O52" t="n">
         <v>4</v>
       </c>
-      <c r="M52" t="n">
-        <v>2</v>
-      </c>
-      <c r="N52" t="n">
-        <v>1</v>
-      </c>
-      <c r="U52" t="n">
+      <c r="P52" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>1</v>
+      </c>
+      <c r="X52" t="n">
         <v>15</v>
       </c>
-      <c r="V52" t="n">
+      <c r="Y52" t="n">
         <v>2388.75</v>
       </c>
     </row>
@@ -3075,44 +3621,47 @@
           <t>WSCR89</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>WSCR89TN</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>WSCR89TN</t>
         </is>
       </c>
-      <c r="G53" t="n">
+      <c r="G53" s="2" t="n"/>
+      <c r="H53" s="2" t="n"/>
+      <c r="I53" s="2" t="n"/>
+      <c r="J53" t="n">
         <v>161.58</v>
       </c>
-      <c r="H53" t="n">
-        <v>1</v>
-      </c>
-      <c r="I53" t="n">
-        <v>1</v>
-      </c>
-      <c r="J53" t="n">
-        <v>3</v>
-      </c>
       <c r="K53" t="n">
+        <v>1</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1</v>
+      </c>
+      <c r="M53" t="n">
+        <v>3</v>
+      </c>
+      <c r="N53" t="n">
         <v>4</v>
       </c>
-      <c r="L53" t="n">
+      <c r="O53" t="n">
         <v>4</v>
       </c>
-      <c r="M53" t="n">
-        <v>2</v>
-      </c>
-      <c r="N53" t="n">
-        <v>1</v>
-      </c>
-      <c r="U53" t="n">
+      <c r="P53" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>1</v>
+      </c>
+      <c r="X53" t="n">
         <v>15</v>
       </c>
-      <c r="V53" t="n">
+      <c r="Y53" t="n">
         <v>2423.7</v>
       </c>
     </row>
@@ -3133,47 +3682,50 @@
           <t>SAF126</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>SAF126BK</t>
         </is>
       </c>
-      <c r="G54" t="n">
+      <c r="G54" s="2" t="n"/>
+      <c r="H54" s="2" t="n"/>
+      <c r="I54" s="2" t="n"/>
+      <c r="J54" t="n">
         <v>135.3</v>
       </c>
-      <c r="H54" t="n">
-        <v>1</v>
-      </c>
-      <c r="M54" t="n">
-        <v>1</v>
-      </c>
-      <c r="N54" t="n">
-        <v>3</v>
-      </c>
-      <c r="O54" t="n">
+      <c r="K54" t="n">
+        <v>1</v>
+      </c>
+      <c r="P54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>3</v>
+      </c>
+      <c r="R54" t="n">
         <v>4</v>
       </c>
-      <c r="P54" t="n">
+      <c r="S54" t="n">
         <v>4</v>
       </c>
-      <c r="Q54" t="n">
-        <v>3</v>
-      </c>
-      <c r="R54" t="n">
-        <v>2</v>
-      </c>
-      <c r="S54" t="n">
-        <v>1</v>
+      <c r="T54" t="n">
+        <v>3</v>
       </c>
       <c r="U54" t="n">
+        <v>2</v>
+      </c>
+      <c r="V54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X54" t="n">
         <v>18</v>
       </c>
-      <c r="V54" t="n">
+      <c r="Y54" t="n">
         <v>2435.4</v>
       </c>
     </row>
@@ -3204,37 +3756,52 @@
           <t>SRF025MR</t>
         </is>
       </c>
-      <c r="G55" t="n">
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>VERAO</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
         <v>153.55</v>
       </c>
-      <c r="H55" t="n">
-        <v>1</v>
-      </c>
-      <c r="M55" t="n">
-        <v>1</v>
-      </c>
-      <c r="N55" t="n">
-        <v>3</v>
-      </c>
-      <c r="O55" t="n">
-        <v>3</v>
+      <c r="K55" t="n">
+        <v>1</v>
       </c>
       <c r="P55" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S55" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="T55" t="n">
+        <v>2</v>
       </c>
       <c r="U55" t="n">
+        <v>2</v>
+      </c>
+      <c r="V55" t="n">
+        <v>1</v>
+      </c>
+      <c r="X55" t="n">
         <v>15</v>
       </c>
-      <c r="V55" t="n">
+      <c r="Y55" t="n">
         <v>2303.25</v>
       </c>
     </row>
@@ -3255,47 +3822,50 @@
           <t>SRT028</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>SRT028BK</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>SRT028BK</t>
         </is>
       </c>
-      <c r="G56" t="n">
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" t="n">
         <v>159.78</v>
       </c>
-      <c r="H56" t="n">
-        <v>1</v>
-      </c>
-      <c r="M56" t="n">
-        <v>1</v>
-      </c>
-      <c r="N56" t="n">
-        <v>3</v>
-      </c>
-      <c r="O56" t="n">
+      <c r="K56" t="n">
+        <v>1</v>
+      </c>
+      <c r="P56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>3</v>
+      </c>
+      <c r="R56" t="n">
         <v>4</v>
       </c>
-      <c r="P56" t="n">
+      <c r="S56" t="n">
         <v>4</v>
       </c>
-      <c r="Q56" t="n">
-        <v>3</v>
-      </c>
-      <c r="R56" t="n">
-        <v>2</v>
-      </c>
-      <c r="S56" t="n">
-        <v>1</v>
+      <c r="T56" t="n">
+        <v>3</v>
       </c>
       <c r="U56" t="n">
+        <v>2</v>
+      </c>
+      <c r="V56" t="n">
+        <v>1</v>
+      </c>
+      <c r="X56" t="n">
         <v>18</v>
       </c>
-      <c r="V56" t="n">
+      <c r="Y56" t="n">
         <v>2876.04</v>
       </c>
     </row>
@@ -3326,31 +3896,46 @@
           <t>SVS027CM</t>
         </is>
       </c>
-      <c r="G57" t="n">
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
         <v>145.11</v>
       </c>
-      <c r="H57" t="n">
-        <v>1</v>
-      </c>
-      <c r="M57" t="n">
-        <v>1</v>
-      </c>
-      <c r="N57" t="n">
-        <v>2</v>
-      </c>
-      <c r="O57" t="n">
-        <v>3</v>
+      <c r="K57" t="n">
+        <v>1</v>
       </c>
       <c r="P57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q57" t="n">
-        <v>3</v>
-      </c>
-      <c r="U57" t="n">
+        <v>2</v>
+      </c>
+      <c r="R57" t="n">
+        <v>3</v>
+      </c>
+      <c r="S57" t="n">
+        <v>3</v>
+      </c>
+      <c r="T57" t="n">
+        <v>3</v>
+      </c>
+      <c r="X57" t="n">
         <v>12</v>
       </c>
-      <c r="V57" t="n">
+      <c r="Y57" t="n">
         <v>1741.32</v>
       </c>
     </row>
@@ -3381,34 +3966,49 @@
           <t>WSC003OW</t>
         </is>
       </c>
-      <c r="G58" t="n">
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TENIS</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
         <v>138.2</v>
       </c>
-      <c r="H58" t="n">
-        <v>1</v>
-      </c>
-      <c r="I58" t="n">
-        <v>1</v>
-      </c>
-      <c r="J58" t="n">
-        <v>1</v>
-      </c>
       <c r="K58" t="n">
+        <v>1</v>
+      </c>
+      <c r="L58" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" t="n">
+        <v>1</v>
+      </c>
+      <c r="N58" t="n">
         <v>4</v>
       </c>
-      <c r="L58" t="n">
+      <c r="O58" t="n">
         <v>5</v>
       </c>
-      <c r="M58" t="n">
-        <v>3</v>
-      </c>
-      <c r="N58" t="n">
-        <v>1</v>
-      </c>
-      <c r="U58" t="n">
+      <c r="P58" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>1</v>
+      </c>
+      <c r="X58" t="n">
         <v>15</v>
       </c>
-      <c r="V58" t="n">
+      <c r="Y58" t="n">
         <v>2073</v>
       </c>
     </row>
@@ -3439,19 +4039,34 @@
           <t>HCT173CF</t>
         </is>
       </c>
-      <c r="G59" t="n">
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>CARTEIRA</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
         <v>52.89</v>
       </c>
-      <c r="H59" t="n">
-        <v>1</v>
-      </c>
-      <c r="T59" t="n">
+      <c r="K59" t="n">
+        <v>1</v>
+      </c>
+      <c r="W59" t="n">
         <v>9</v>
       </c>
-      <c r="U59" t="n">
+      <c r="X59" t="n">
         <v>9</v>
       </c>
-      <c r="V59" t="n">
+      <c r="Y59" t="n">
         <v>476.01</v>
       </c>
     </row>
@@ -3482,19 +4097,34 @@
           <t>HCT173PT</t>
         </is>
       </c>
-      <c r="G60" t="n">
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>CARTEIRA</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>CLASSICO</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
         <v>52.89</v>
       </c>
-      <c r="H60" t="n">
-        <v>1</v>
-      </c>
-      <c r="T60" t="n">
+      <c r="K60" t="n">
+        <v>1</v>
+      </c>
+      <c r="W60" t="n">
         <v>6</v>
       </c>
-      <c r="U60" t="n">
+      <c r="X60" t="n">
         <v>6</v>
       </c>
-      <c r="V60" t="n">
+      <c r="Y60" t="n">
         <v>317.34</v>
       </c>
     </row>
@@ -3525,19 +4155,34 @@
           <t>MCC008TN</t>
         </is>
       </c>
-      <c r="G61" t="n">
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>COMPLEMENTOS</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
         <v>39.04</v>
       </c>
-      <c r="H61" t="n">
-        <v>1</v>
-      </c>
-      <c r="T61" t="n">
+      <c r="K61" t="n">
+        <v>1</v>
+      </c>
+      <c r="W61" t="n">
         <v>9</v>
       </c>
-      <c r="U61" t="n">
+      <c r="X61" t="n">
         <v>9</v>
       </c>
-      <c r="V61" t="n">
+      <c r="Y61" t="n">
         <v>351.36</v>
       </c>
     </row>
@@ -3568,19 +4213,34 @@
           <t>MCC008VR</t>
         </is>
       </c>
-      <c r="G62" t="n">
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>ACESSORIOS</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>COMPLEMENTOS</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
         <v>39.04</v>
       </c>
-      <c r="H62" t="n">
-        <v>1</v>
-      </c>
-      <c r="T62" t="n">
+      <c r="K62" t="n">
+        <v>1</v>
+      </c>
+      <c r="W62" t="n">
         <v>9</v>
       </c>
-      <c r="U62" t="n">
+      <c r="X62" t="n">
         <v>9</v>
       </c>
-      <c r="V62" t="n">
+      <c r="Y62" t="n">
         <v>351.36</v>
       </c>
     </row>
@@ -3611,34 +4271,49 @@
           <t>PRA127CF</t>
         </is>
       </c>
-      <c r="G63" t="n">
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>SANDALIA RASTEIRA</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>INVERNO</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
         <v>61.13</v>
       </c>
-      <c r="H63" t="n">
-        <v>1</v>
-      </c>
-      <c r="I63" t="n">
-        <v>1</v>
-      </c>
-      <c r="J63" t="n">
-        <v>3</v>
-      </c>
       <c r="K63" t="n">
+        <v>1</v>
+      </c>
+      <c r="L63" t="n">
+        <v>1</v>
+      </c>
+      <c r="M63" t="n">
+        <v>3</v>
+      </c>
+      <c r="N63" t="n">
         <v>4</v>
       </c>
-      <c r="L63" t="n">
-        <v>3</v>
-      </c>
-      <c r="M63" t="n">
-        <v>3</v>
-      </c>
-      <c r="N63" t="n">
-        <v>1</v>
-      </c>
-      <c r="U63" t="n">
+      <c r="O63" t="n">
+        <v>3</v>
+      </c>
+      <c r="P63" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>1</v>
+      </c>
+      <c r="X63" t="n">
         <v>15</v>
       </c>
-      <c r="V63" t="n">
+      <c r="Y63" t="n">
         <v>916.95</v>
       </c>
     </row>
@@ -3659,44 +4334,47 @@
           <t>PRA728</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>PRA728FD</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>PRA728FD</t>
         </is>
       </c>
-      <c r="G64" t="n">
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="n"/>
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" t="n">
         <v>70.93000000000001</v>
       </c>
-      <c r="H64" t="n">
-        <v>1</v>
-      </c>
-      <c r="I64" t="n">
-        <v>1</v>
-      </c>
-      <c r="J64" t="n">
-        <v>3</v>
-      </c>
       <c r="K64" t="n">
+        <v>1</v>
+      </c>
+      <c r="L64" t="n">
+        <v>1</v>
+      </c>
+      <c r="M64" t="n">
+        <v>3</v>
+      </c>
+      <c r="N64" t="n">
         <v>4</v>
       </c>
-      <c r="L64" t="n">
-        <v>3</v>
-      </c>
-      <c r="M64" t="n">
-        <v>3</v>
-      </c>
-      <c r="N64" t="n">
-        <v>1</v>
-      </c>
-      <c r="U64" t="n">
+      <c r="O64" t="n">
+        <v>3</v>
+      </c>
+      <c r="P64" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>1</v>
+      </c>
+      <c r="X64" t="n">
         <v>15</v>
       </c>
-      <c r="V64" t="n">
+      <c r="Y64" t="n">
         <v>1063.95</v>
       </c>
     </row>
@@ -3717,44 +4395,47 @@
           <t>PRA728</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>PRA728VO</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>PRA728VO</t>
         </is>
       </c>
-      <c r="G65" t="n">
+      <c r="G65" s="2" t="n"/>
+      <c r="H65" s="2" t="n"/>
+      <c r="I65" s="2" t="n"/>
+      <c r="J65" t="n">
         <v>70.93000000000001</v>
       </c>
-      <c r="H65" t="n">
-        <v>1</v>
-      </c>
-      <c r="I65" t="n">
-        <v>1</v>
-      </c>
-      <c r="J65" t="n">
-        <v>2</v>
-      </c>
       <c r="K65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M65" t="n">
         <v>2</v>
       </c>
       <c r="N65" t="n">
-        <v>1</v>
-      </c>
-      <c r="U65" t="n">
+        <v>3</v>
+      </c>
+      <c r="O65" t="n">
+        <v>3</v>
+      </c>
+      <c r="P65" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>1</v>
+      </c>
+      <c r="X65" t="n">
         <v>12</v>
       </c>
-      <c r="V65" t="n">
+      <c r="Y65" t="n">
         <v>851.16</v>
       </c>
     </row>
@@ -3775,44 +4456,47 @@
           <t>TBC207</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>TBC207CA</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>TBC207CA</t>
         </is>
       </c>
-      <c r="G66" t="n">
+      <c r="G66" s="2" t="n"/>
+      <c r="H66" s="2" t="n"/>
+      <c r="I66" s="2" t="n"/>
+      <c r="J66" t="n">
         <v>56.96</v>
       </c>
-      <c r="H66" t="n">
-        <v>1</v>
-      </c>
-      <c r="I66" t="n">
-        <v>1</v>
-      </c>
-      <c r="J66" t="n">
-        <v>3</v>
-      </c>
       <c r="K66" t="n">
+        <v>1</v>
+      </c>
+      <c r="L66" t="n">
+        <v>1</v>
+      </c>
+      <c r="M66" t="n">
+        <v>3</v>
+      </c>
+      <c r="N66" t="n">
         <v>5</v>
       </c>
-      <c r="L66" t="n">
+      <c r="O66" t="n">
         <v>4</v>
       </c>
-      <c r="M66" t="n">
-        <v>3</v>
-      </c>
-      <c r="N66" t="n">
-        <v>2</v>
-      </c>
-      <c r="U66" t="n">
+      <c r="P66" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>2</v>
+      </c>
+      <c r="X66" t="n">
         <v>18</v>
       </c>
-      <c r="V66" t="n">
+      <c r="Y66" t="n">
         <v>1025.28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add price pyramid to unified spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9PfgDEdKqrS7U5PG39u7r
</commit_message>
<xml_diff>
--- a/pedidos/Pedidos_Nova_America_Unificado.xlsx
+++ b/pedidos/Pedidos_Nova_America_Unificado.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y66"/>
+  <dimension ref="A1:AA66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,58 +475,68 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Preço</t>
+          <t>Preço Venda</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Pirâmide</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Preço Pedido</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Qtd Caixas</t>
         </is>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="N1" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="O1" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="P1" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="Q1" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="R1" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="S1" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="T1" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="U1" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="T1" s="1" t="n">
+      <c r="V1" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="U1" s="1" t="n">
+      <c r="W1" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="X1" s="1" t="n">
         <v>44</v>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>UN</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Qtd Total</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Vlr Total</t>
         </is>
@@ -562,37 +572,39 @@
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
-      <c r="J2" t="n">
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" t="n">
         <v>268.14</v>
       </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>2</v>
+      <c r="M2" t="n">
+        <v>1</v>
       </c>
       <c r="R2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T2" t="n">
         <v>3</v>
       </c>
       <c r="U2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V2" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="W2" t="n">
+        <v>2</v>
       </c>
       <c r="X2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z2" t="n">
         <v>15</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AA2" t="n">
         <v>4022.1</v>
       </c>
     </row>
@@ -639,36 +651,44 @@
         </is>
       </c>
       <c r="J3" t="n">
+        <v>599.9</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
         <v>209.1</v>
       </c>
-      <c r="K3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>2</v>
+      <c r="M3" t="n">
+        <v>1</v>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
+        <v>2</v>
+      </c>
+      <c r="T3" t="n">
+        <v>3</v>
+      </c>
+      <c r="U3" t="n">
         <v>4</v>
       </c>
-      <c r="T3" t="n">
-        <v>3</v>
-      </c>
-      <c r="U3" t="n">
-        <v>1</v>
-      </c>
       <c r="V3" t="n">
+        <v>3</v>
+      </c>
+      <c r="W3" t="n">
         <v>1</v>
       </c>
       <c r="X3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z3" t="n">
         <v>15</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="AA3" t="n">
         <v>3136.5</v>
       </c>
     </row>
@@ -702,37 +722,39 @@
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
-      <c r="J4" t="n">
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" t="n">
         <v>242.31</v>
       </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>2</v>
+      <c r="M4" t="n">
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T4" t="n">
         <v>3</v>
       </c>
       <c r="U4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V4" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="W4" t="n">
+        <v>2</v>
       </c>
       <c r="X4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z4" t="n">
         <v>15</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="AA4" t="n">
         <v>3634.65</v>
       </c>
     </row>
@@ -779,21 +801,29 @@
         </is>
       </c>
       <c r="J5" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
         <v>19.91</v>
       </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
         <v>12</v>
       </c>
-      <c r="R5" t="n">
+      <c r="T5" t="n">
         <v>12</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Z5" t="n">
         <v>24</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="AA5" t="n">
         <v>477.84</v>
       </c>
     </row>
@@ -840,21 +870,29 @@
         </is>
       </c>
       <c r="J6" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
         <v>19.91</v>
       </c>
-      <c r="K6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
         <v>24</v>
       </c>
-      <c r="R6" t="n">
+      <c r="T6" t="n">
         <v>24</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Z6" t="n">
         <v>48</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="AA6" t="n">
         <v>955.6799999999999</v>
       </c>
     </row>
@@ -888,34 +926,36 @@
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
-      <c r="J7" t="n">
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" t="n">
         <v>54.9</v>
       </c>
-      <c r="K7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" t="n">
-        <v>1</v>
-      </c>
       <c r="M7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
-      </c>
-      <c r="X7" t="n">
+        <v>3</v>
+      </c>
+      <c r="R7" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" t="n">
         <v>12</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="AA7" t="n">
         <v>658.8</v>
       </c>
     </row>
@@ -949,34 +989,36 @@
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
-      <c r="J8" t="n">
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" t="n">
         <v>60.88</v>
       </c>
-      <c r="K8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" t="n">
-        <v>1</v>
-      </c>
       <c r="M8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" t="n">
         <v>4</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>4</v>
       </c>
-      <c r="P8" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>1</v>
-      </c>
-      <c r="X8" t="n">
+      <c r="R8" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z8" t="n">
         <v>15</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="AA8" t="n">
         <v>913.2</v>
       </c>
     </row>
@@ -1010,34 +1052,36 @@
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
-      <c r="J9" t="n">
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" t="n">
         <v>60.88</v>
       </c>
-      <c r="K9" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" t="n">
-        <v>1</v>
-      </c>
       <c r="M9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>3</v>
+      </c>
+      <c r="P9" t="n">
         <v>4</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>4</v>
       </c>
-      <c r="P9" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>1</v>
-      </c>
-      <c r="X9" t="n">
+      <c r="R9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z9" t="n">
         <v>15</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="AA9" t="n">
         <v>913.2</v>
       </c>
     </row>
@@ -1071,34 +1115,36 @@
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
-      <c r="J10" t="n">
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" t="n">
         <v>60.88</v>
       </c>
-      <c r="K10" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
       <c r="M10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" t="n">
         <v>4</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>4</v>
       </c>
-      <c r="P10" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>1</v>
-      </c>
-      <c r="X10" t="n">
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z10" t="n">
         <v>15</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="AA10" t="n">
         <v>913.2</v>
       </c>
     </row>
@@ -1132,34 +1178,36 @@
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
-      <c r="J11" t="n">
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" t="n">
         <v>60.88</v>
       </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
       <c r="M11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>3</v>
+      </c>
+      <c r="P11" t="n">
         <v>4</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>4</v>
       </c>
-      <c r="P11" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>1</v>
-      </c>
-      <c r="X11" t="n">
+      <c r="R11" t="n">
+        <v>2</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z11" t="n">
         <v>15</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AA11" t="n">
         <v>913.2</v>
       </c>
     </row>
@@ -1206,18 +1254,26 @@
         </is>
       </c>
       <c r="J12" t="n">
+        <v>669.9</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
         <v>230.4</v>
       </c>
-      <c r="K12" t="n">
-        <v>1</v>
-      </c>
-      <c r="W12" t="n">
-        <v>2</v>
-      </c>
-      <c r="X12" t="n">
-        <v>2</v>
+      <c r="M12" t="n">
+        <v>1</v>
       </c>
       <c r="Y12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA12" t="n">
         <v>460.8</v>
       </c>
     </row>
@@ -1264,18 +1320,26 @@
         </is>
       </c>
       <c r="J13" t="n">
+        <v>599.9</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
         <v>234</v>
       </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="W13" t="n">
-        <v>3</v>
-      </c>
-      <c r="X13" t="n">
-        <v>3</v>
+      <c r="M13" t="n">
+        <v>1</v>
       </c>
       <c r="Y13" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA13" t="n">
         <v>702</v>
       </c>
     </row>
@@ -1322,18 +1386,26 @@
         </is>
       </c>
       <c r="J14" t="n">
+        <v>699.9</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
         <v>240</v>
       </c>
-      <c r="K14" t="n">
-        <v>1</v>
-      </c>
-      <c r="W14" t="n">
-        <v>1</v>
-      </c>
-      <c r="X14" t="n">
+      <c r="M14" t="n">
         <v>1</v>
       </c>
       <c r="Y14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA14" t="n">
         <v>240</v>
       </c>
     </row>
@@ -1380,18 +1452,26 @@
         </is>
       </c>
       <c r="J15" t="n">
+        <v>699.9</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
         <v>240</v>
       </c>
-      <c r="K15" t="n">
-        <v>1</v>
-      </c>
-      <c r="W15" t="n">
-        <v>1</v>
-      </c>
-      <c r="X15" t="n">
+      <c r="M15" t="n">
         <v>1</v>
       </c>
       <c r="Y15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA15" t="n">
         <v>240</v>
       </c>
     </row>
@@ -1425,34 +1505,36 @@
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
-      <c r="J16" t="n">
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" t="n">
         <v>149.31</v>
       </c>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" t="n">
-        <v>1</v>
-      </c>
       <c r="M16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q16" t="n">
-        <v>1</v>
-      </c>
-      <c r="X16" t="n">
+        <v>3</v>
+      </c>
+      <c r="R16" t="n">
+        <v>2</v>
+      </c>
+      <c r="S16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z16" t="n">
         <v>12</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="AA16" t="n">
         <v>1791.72</v>
       </c>
     </row>
@@ -1486,34 +1568,36 @@
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
-      <c r="J17" t="n">
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" t="n">
         <v>145.33</v>
       </c>
-      <c r="K17" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1</v>
-      </c>
       <c r="M17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q17" t="n">
-        <v>1</v>
-      </c>
-      <c r="X17" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" t="n">
+        <v>2</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z17" t="n">
         <v>12</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="AA17" t="n">
         <v>1743.96</v>
       </c>
     </row>
@@ -1547,34 +1631,36 @@
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
-      <c r="J18" t="n">
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" t="n">
         <v>154.12</v>
       </c>
-      <c r="K18" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" t="n">
-        <v>1</v>
-      </c>
       <c r="M18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q18" t="n">
-        <v>1</v>
-      </c>
-      <c r="X18" t="n">
+        <v>3</v>
+      </c>
+      <c r="R18" t="n">
+        <v>2</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z18" t="n">
         <v>12</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="AA18" t="n">
         <v>1849.44</v>
       </c>
     </row>
@@ -1608,34 +1694,36 @@
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
-      <c r="J19" t="n">
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" t="n">
         <v>68.31999999999999</v>
       </c>
-      <c r="K19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" t="n">
-        <v>1</v>
-      </c>
       <c r="M19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>3</v>
+      </c>
+      <c r="P19" t="n">
         <v>4</v>
       </c>
-      <c r="O19" t="n">
+      <c r="Q19" t="n">
         <v>5</v>
       </c>
-      <c r="P19" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>2</v>
-      </c>
-      <c r="X19" t="n">
+      <c r="R19" t="n">
+        <v>3</v>
+      </c>
+      <c r="S19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z19" t="n">
         <v>18</v>
       </c>
-      <c r="Y19" t="n">
+      <c r="AA19" t="n">
         <v>1229.76</v>
       </c>
     </row>
@@ -1682,33 +1770,41 @@
         </is>
       </c>
       <c r="J20" t="n">
+        <v>399.9</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
         <v>118.83</v>
       </c>
-      <c r="K20" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" t="n">
-        <v>1</v>
-      </c>
       <c r="M20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N20" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>3</v>
+      </c>
+      <c r="P20" t="n">
         <v>4</v>
       </c>
-      <c r="O20" t="n">
+      <c r="Q20" t="n">
         <v>6</v>
       </c>
-      <c r="P20" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>2</v>
-      </c>
-      <c r="X20" t="n">
+      <c r="R20" t="n">
+        <v>2</v>
+      </c>
+      <c r="S20" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z20" t="n">
         <v>18</v>
       </c>
-      <c r="Y20" t="n">
+      <c r="AA20" t="n">
         <v>2138.94</v>
       </c>
     </row>
@@ -1755,33 +1851,41 @@
         </is>
       </c>
       <c r="J21" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
         <v>109.2</v>
       </c>
-      <c r="K21" t="n">
-        <v>1</v>
-      </c>
-      <c r="L21" t="n">
-        <v>1</v>
-      </c>
       <c r="M21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N21" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>3</v>
+      </c>
+      <c r="P21" t="n">
         <v>4</v>
       </c>
-      <c r="O21" t="n">
+      <c r="Q21" t="n">
         <v>4</v>
       </c>
-      <c r="P21" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>1</v>
-      </c>
-      <c r="X21" t="n">
+      <c r="R21" t="n">
+        <v>2</v>
+      </c>
+      <c r="S21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z21" t="n">
         <v>15</v>
       </c>
-      <c r="Y21" t="n">
+      <c r="AA21" t="n">
         <v>1638</v>
       </c>
     </row>
@@ -1815,34 +1919,36 @@
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
-      <c r="J22" t="n">
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" t="n">
         <v>110.18</v>
       </c>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" t="n">
-        <v>1</v>
-      </c>
       <c r="M22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>3</v>
+      </c>
+      <c r="P22" t="n">
         <v>4</v>
       </c>
-      <c r="O22" t="n">
+      <c r="Q22" t="n">
         <v>4</v>
       </c>
-      <c r="P22" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>1</v>
-      </c>
-      <c r="X22" t="n">
+      <c r="R22" t="n">
+        <v>2</v>
+      </c>
+      <c r="S22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z22" t="n">
         <v>15</v>
       </c>
-      <c r="Y22" t="n">
+      <c r="AA22" t="n">
         <v>1652.7</v>
       </c>
     </row>
@@ -1876,34 +1982,36 @@
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
-      <c r="J23" t="n">
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" t="n">
         <v>61.35</v>
       </c>
-      <c r="K23" t="n">
-        <v>1</v>
-      </c>
-      <c r="L23" t="n">
-        <v>1</v>
-      </c>
       <c r="M23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>3</v>
+      </c>
+      <c r="P23" t="n">
         <v>4</v>
       </c>
-      <c r="O23" t="n">
-        <v>3</v>
-      </c>
-      <c r="P23" t="n">
-        <v>3</v>
-      </c>
       <c r="Q23" t="n">
-        <v>1</v>
-      </c>
-      <c r="X23" t="n">
+        <v>3</v>
+      </c>
+      <c r="R23" t="n">
+        <v>3</v>
+      </c>
+      <c r="S23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z23" t="n">
         <v>15</v>
       </c>
-      <c r="Y23" t="n">
+      <c r="AA23" t="n">
         <v>920.25</v>
       </c>
     </row>
@@ -1950,18 +2058,26 @@
         </is>
       </c>
       <c r="J24" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
         <v>17.51</v>
       </c>
-      <c r="K24" t="n">
-        <v>1</v>
-      </c>
-      <c r="W24" t="n">
+      <c r="M24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y24" t="n">
         <v>24</v>
       </c>
-      <c r="X24" t="n">
+      <c r="Z24" t="n">
         <v>24</v>
       </c>
-      <c r="Y24" t="n">
+      <c r="AA24" t="n">
         <v>420.24</v>
       </c>
     </row>
@@ -2008,18 +2124,26 @@
         </is>
       </c>
       <c r="J25" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
         <v>17.51</v>
       </c>
-      <c r="K25" t="n">
-        <v>1</v>
-      </c>
-      <c r="W25" t="n">
+      <c r="M25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y25" t="n">
         <v>24</v>
       </c>
-      <c r="X25" t="n">
+      <c r="Z25" t="n">
         <v>24</v>
       </c>
-      <c r="Y25" t="n">
+      <c r="AA25" t="n">
         <v>420.24</v>
       </c>
     </row>
@@ -2066,18 +2190,26 @@
         </is>
       </c>
       <c r="J26" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
         <v>17.51</v>
       </c>
-      <c r="K26" t="n">
-        <v>1</v>
-      </c>
-      <c r="W26" t="n">
+      <c r="M26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y26" t="n">
         <v>36</v>
       </c>
-      <c r="X26" t="n">
+      <c r="Z26" t="n">
         <v>36</v>
       </c>
-      <c r="Y26" t="n">
+      <c r="AA26" t="n">
         <v>630.36</v>
       </c>
     </row>
@@ -2124,18 +2256,26 @@
         </is>
       </c>
       <c r="J27" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
         <v>15.63</v>
       </c>
-      <c r="K27" t="n">
-        <v>1</v>
-      </c>
-      <c r="W27" t="n">
+      <c r="M27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y27" t="n">
         <v>36</v>
       </c>
-      <c r="X27" t="n">
+      <c r="Z27" t="n">
         <v>36</v>
       </c>
-      <c r="Y27" t="n">
+      <c r="AA27" t="n">
         <v>562.6799999999999</v>
       </c>
     </row>
@@ -2182,18 +2322,26 @@
         </is>
       </c>
       <c r="J28" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
         <v>15.33</v>
       </c>
-      <c r="K28" t="n">
-        <v>1</v>
-      </c>
-      <c r="W28" t="n">
+      <c r="M28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y28" t="n">
         <v>60</v>
       </c>
-      <c r="X28" t="n">
+      <c r="Z28" t="n">
         <v>60</v>
       </c>
-      <c r="Y28" t="n">
+      <c r="AA28" t="n">
         <v>919.8</v>
       </c>
     </row>
@@ -2240,18 +2388,26 @@
         </is>
       </c>
       <c r="J29" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
         <v>15.33</v>
       </c>
-      <c r="K29" t="n">
-        <v>1</v>
-      </c>
-      <c r="W29" t="n">
+      <c r="M29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y29" t="n">
         <v>36</v>
       </c>
-      <c r="X29" t="n">
+      <c r="Z29" t="n">
         <v>36</v>
       </c>
-      <c r="Y29" t="n">
+      <c r="AA29" t="n">
         <v>551.88</v>
       </c>
     </row>
@@ -2298,18 +2454,26 @@
         </is>
       </c>
       <c r="J30" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
         <v>15.33</v>
       </c>
-      <c r="K30" t="n">
-        <v>1</v>
-      </c>
-      <c r="W30" t="n">
+      <c r="M30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y30" t="n">
         <v>60</v>
       </c>
-      <c r="X30" t="n">
+      <c r="Z30" t="n">
         <v>60</v>
       </c>
-      <c r="Y30" t="n">
+      <c r="AA30" t="n">
         <v>919.8</v>
       </c>
     </row>
@@ -2343,19 +2507,21 @@
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
-      <c r="J31" t="n">
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" t="n">
         <v>242.99</v>
       </c>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
-      <c r="W31" t="n">
-        <v>2</v>
-      </c>
-      <c r="X31" t="n">
-        <v>2</v>
+      <c r="M31" t="n">
+        <v>1</v>
       </c>
       <c r="Y31" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA31" t="n">
         <v>485.98</v>
       </c>
     </row>
@@ -2389,19 +2555,21 @@
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
-      <c r="J32" t="n">
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" t="n">
         <v>242.99</v>
       </c>
-      <c r="K32" t="n">
-        <v>1</v>
-      </c>
-      <c r="W32" t="n">
-        <v>2</v>
-      </c>
-      <c r="X32" t="n">
-        <v>2</v>
+      <c r="M32" t="n">
+        <v>1</v>
       </c>
       <c r="Y32" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA32" t="n">
         <v>485.98</v>
       </c>
     </row>
@@ -2435,19 +2603,21 @@
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
-      <c r="J33" t="n">
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" t="n">
         <v>235</v>
       </c>
-      <c r="K33" t="n">
-        <v>1</v>
-      </c>
-      <c r="W33" t="n">
-        <v>2</v>
-      </c>
-      <c r="X33" t="n">
-        <v>2</v>
+      <c r="M33" t="n">
+        <v>1</v>
       </c>
       <c r="Y33" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA33" t="n">
         <v>470</v>
       </c>
     </row>
@@ -2494,18 +2664,26 @@
         </is>
       </c>
       <c r="J34" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
         <v>122.67</v>
       </c>
-      <c r="K34" t="n">
-        <v>1</v>
-      </c>
-      <c r="W34" t="n">
-        <v>2</v>
-      </c>
-      <c r="X34" t="n">
-        <v>2</v>
+      <c r="M34" t="n">
+        <v>1</v>
       </c>
       <c r="Y34" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA34" t="n">
         <v>245.34</v>
       </c>
     </row>
@@ -2552,18 +2730,26 @@
         </is>
       </c>
       <c r="J35" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
         <v>122.67</v>
       </c>
-      <c r="K35" t="n">
-        <v>1</v>
-      </c>
-      <c r="W35" t="n">
-        <v>3</v>
-      </c>
-      <c r="X35" t="n">
-        <v>3</v>
+      <c r="M35" t="n">
+        <v>1</v>
       </c>
       <c r="Y35" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA35" t="n">
         <v>368.01</v>
       </c>
     </row>
@@ -2597,19 +2783,21 @@
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="n"/>
-      <c r="J36" t="n">
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" t="n">
         <v>200.69</v>
       </c>
-      <c r="K36" t="n">
-        <v>1</v>
-      </c>
-      <c r="W36" t="n">
-        <v>2</v>
-      </c>
-      <c r="X36" t="n">
-        <v>2</v>
+      <c r="M36" t="n">
+        <v>1</v>
       </c>
       <c r="Y36" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA36" t="n">
         <v>401.38</v>
       </c>
     </row>
@@ -2643,19 +2831,21 @@
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="n"/>
-      <c r="J37" t="n">
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" t="n">
         <v>138.06</v>
       </c>
-      <c r="K37" t="n">
-        <v>1</v>
-      </c>
-      <c r="W37" t="n">
-        <v>3</v>
-      </c>
-      <c r="X37" t="n">
-        <v>3</v>
+      <c r="M37" t="n">
+        <v>1</v>
       </c>
       <c r="Y37" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA37" t="n">
         <v>414.18</v>
       </c>
     </row>
@@ -2689,19 +2879,21 @@
       <c r="G38" s="2" t="n"/>
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
-      <c r="J38" t="n">
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" t="n">
         <v>138.06</v>
       </c>
-      <c r="K38" t="n">
-        <v>1</v>
-      </c>
-      <c r="W38" t="n">
-        <v>3</v>
-      </c>
-      <c r="X38" t="n">
-        <v>3</v>
+      <c r="M38" t="n">
+        <v>1</v>
       </c>
       <c r="Y38" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA38" t="n">
         <v>414.18</v>
       </c>
     </row>
@@ -2748,18 +2940,26 @@
         </is>
       </c>
       <c r="J39" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
         <v>85.78</v>
       </c>
-      <c r="K39" t="n">
-        <v>1</v>
-      </c>
-      <c r="W39" t="n">
+      <c r="M39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y39" t="n">
         <v>8</v>
       </c>
-      <c r="X39" t="n">
+      <c r="Z39" t="n">
         <v>8</v>
       </c>
-      <c r="Y39" t="n">
+      <c r="AA39" t="n">
         <v>686.24</v>
       </c>
     </row>
@@ -2806,18 +3006,26 @@
         </is>
       </c>
       <c r="J40" t="n">
+        <v>339.9</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
         <v>122.2</v>
       </c>
-      <c r="K40" t="n">
-        <v>1</v>
-      </c>
-      <c r="W40" t="n">
-        <v>2</v>
-      </c>
-      <c r="X40" t="n">
-        <v>2</v>
+      <c r="M40" t="n">
+        <v>1</v>
       </c>
       <c r="Y40" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA40" t="n">
         <v>244.4</v>
       </c>
     </row>
@@ -2864,18 +3072,26 @@
         </is>
       </c>
       <c r="J41" t="n">
+        <v>339.9</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
         <v>123.38</v>
       </c>
-      <c r="K41" t="n">
-        <v>1</v>
-      </c>
-      <c r="W41" t="n">
+      <c r="M41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y41" t="n">
         <v>4</v>
       </c>
-      <c r="X41" t="n">
+      <c r="Z41" t="n">
         <v>4</v>
       </c>
-      <c r="Y41" t="n">
+      <c r="AA41" t="n">
         <v>493.52</v>
       </c>
     </row>
@@ -2922,18 +3138,26 @@
         </is>
       </c>
       <c r="J42" t="n">
+        <v>339.9</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
         <v>123.38</v>
       </c>
-      <c r="K42" t="n">
-        <v>1</v>
-      </c>
-      <c r="W42" t="n">
+      <c r="M42" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y42" t="n">
         <v>4</v>
       </c>
-      <c r="X42" t="n">
+      <c r="Z42" t="n">
         <v>4</v>
       </c>
-      <c r="Y42" t="n">
+      <c r="AA42" t="n">
         <v>493.52</v>
       </c>
     </row>
@@ -2980,18 +3204,26 @@
         </is>
       </c>
       <c r="J43" t="n">
+        <v>139.9</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
         <v>45.77</v>
       </c>
-      <c r="K43" t="n">
-        <v>1</v>
-      </c>
-      <c r="W43" t="n">
+      <c r="M43" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y43" t="n">
         <v>4</v>
       </c>
-      <c r="X43" t="n">
+      <c r="Z43" t="n">
         <v>4</v>
       </c>
-      <c r="Y43" t="n">
+      <c r="AA43" t="n">
         <v>183.08</v>
       </c>
     </row>
@@ -3038,18 +3270,26 @@
         </is>
       </c>
       <c r="J44" t="n">
+        <v>139.9</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
         <v>45.77</v>
       </c>
-      <c r="K44" t="n">
-        <v>1</v>
-      </c>
-      <c r="W44" t="n">
+      <c r="M44" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y44" t="n">
         <v>9</v>
       </c>
-      <c r="X44" t="n">
+      <c r="Z44" t="n">
         <v>9</v>
       </c>
-      <c r="Y44" t="n">
+      <c r="AA44" t="n">
         <v>411.93</v>
       </c>
     </row>
@@ -3096,18 +3336,26 @@
         </is>
       </c>
       <c r="J45" t="n">
+        <v>149.9</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L45" t="n">
         <v>49.35</v>
       </c>
-      <c r="K45" t="n">
-        <v>1</v>
-      </c>
-      <c r="W45" t="n">
+      <c r="M45" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y45" t="n">
         <v>9</v>
       </c>
-      <c r="X45" t="n">
+      <c r="Z45" t="n">
         <v>9</v>
       </c>
-      <c r="Y45" t="n">
+      <c r="AA45" t="n">
         <v>444.15</v>
       </c>
     </row>
@@ -3154,18 +3402,26 @@
         </is>
       </c>
       <c r="J46" t="n">
+        <v>139.9</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
         <v>45.78</v>
       </c>
-      <c r="K46" t="n">
-        <v>1</v>
-      </c>
-      <c r="W46" t="n">
+      <c r="M46" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y46" t="n">
         <v>6</v>
       </c>
-      <c r="X46" t="n">
+      <c r="Z46" t="n">
         <v>6</v>
       </c>
-      <c r="Y46" t="n">
+      <c r="AA46" t="n">
         <v>274.68</v>
       </c>
     </row>
@@ -3212,33 +3468,41 @@
         </is>
       </c>
       <c r="J47" t="n">
+        <v>369.9</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L47" t="n">
         <v>114.1</v>
       </c>
-      <c r="K47" t="n">
-        <v>1</v>
-      </c>
-      <c r="P47" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>2</v>
+      <c r="M47" t="n">
+        <v>1</v>
       </c>
       <c r="R47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S47" t="n">
+        <v>2</v>
+      </c>
+      <c r="T47" t="n">
+        <v>2</v>
+      </c>
+      <c r="U47" t="n">
         <v>4</v>
       </c>
-      <c r="T47" t="n">
-        <v>2</v>
-      </c>
-      <c r="U47" t="n">
-        <v>1</v>
-      </c>
-      <c r="X47" t="n">
+      <c r="V47" t="n">
+        <v>2</v>
+      </c>
+      <c r="W47" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z47" t="n">
         <v>12</v>
       </c>
-      <c r="Y47" t="n">
+      <c r="AA47" t="n">
         <v>1369.2</v>
       </c>
     </row>
@@ -3285,36 +3549,44 @@
         </is>
       </c>
       <c r="J48" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L48" t="n">
         <v>74.66</v>
       </c>
-      <c r="K48" t="n">
-        <v>1</v>
-      </c>
-      <c r="P48" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>2</v>
+      <c r="M48" t="n">
+        <v>1</v>
       </c>
       <c r="R48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T48" t="n">
         <v>3</v>
       </c>
       <c r="U48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V48" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="W48" t="n">
+        <v>2</v>
       </c>
       <c r="X48" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z48" t="n">
         <v>15</v>
       </c>
-      <c r="Y48" t="n">
+      <c r="AA48" t="n">
         <v>1119.9</v>
       </c>
     </row>
@@ -3361,33 +3633,41 @@
         </is>
       </c>
       <c r="J49" t="n">
+        <v>599.9</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L49" t="n">
         <v>200.54</v>
       </c>
-      <c r="K49" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>2</v>
-      </c>
-      <c r="R49" t="n">
-        <v>3</v>
+      <c r="M49" t="n">
+        <v>1</v>
       </c>
       <c r="S49" t="n">
+        <v>2</v>
+      </c>
+      <c r="T49" t="n">
+        <v>3</v>
+      </c>
+      <c r="U49" t="n">
         <v>4</v>
       </c>
-      <c r="T49" t="n">
+      <c r="V49" t="n">
         <v>4</v>
       </c>
-      <c r="U49" t="n">
-        <v>3</v>
-      </c>
-      <c r="V49" t="n">
-        <v>2</v>
+      <c r="W49" t="n">
+        <v>3</v>
       </c>
       <c r="X49" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z49" t="n">
         <v>18</v>
       </c>
-      <c r="Y49" t="n">
+      <c r="AA49" t="n">
         <v>3609.72</v>
       </c>
     </row>
@@ -3434,36 +3714,44 @@
         </is>
       </c>
       <c r="J50" t="n">
+        <v>599.9</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
         <v>200.54</v>
       </c>
-      <c r="K50" t="n">
-        <v>1</v>
-      </c>
-      <c r="P50" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q50" t="n">
+      <c r="M50" t="n">
         <v>1</v>
       </c>
       <c r="R50" t="n">
+        <v>1</v>
+      </c>
+      <c r="S50" t="n">
+        <v>1</v>
+      </c>
+      <c r="T50" t="n">
         <v>4</v>
       </c>
-      <c r="S50" t="n">
+      <c r="U50" t="n">
         <v>4</v>
       </c>
-      <c r="T50" t="n">
-        <v>3</v>
-      </c>
-      <c r="U50" t="n">
-        <v>1</v>
-      </c>
       <c r="V50" t="n">
+        <v>3</v>
+      </c>
+      <c r="W50" t="n">
         <v>1</v>
       </c>
       <c r="X50" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z50" t="n">
         <v>15</v>
       </c>
-      <c r="Y50" t="n">
+      <c r="AA50" t="n">
         <v>3008.1</v>
       </c>
     </row>
@@ -3510,36 +3798,44 @@
         </is>
       </c>
       <c r="J51" t="n">
+        <v>539.9</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L51" t="n">
         <v>183.09</v>
       </c>
-      <c r="K51" t="n">
-        <v>1</v>
-      </c>
-      <c r="P51" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>2</v>
+      <c r="M51" t="n">
+        <v>1</v>
       </c>
       <c r="R51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V51" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="W51" t="n">
+        <v>2</v>
       </c>
       <c r="X51" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z51" t="n">
         <v>14</v>
       </c>
-      <c r="Y51" t="n">
+      <c r="AA51" t="n">
         <v>2563.26</v>
       </c>
     </row>
@@ -3573,34 +3869,36 @@
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="n"/>
-      <c r="J52" t="n">
+      <c r="J52" s="2" t="n"/>
+      <c r="K52" s="2" t="n"/>
+      <c r="L52" t="n">
         <v>159.25</v>
       </c>
-      <c r="K52" t="n">
-        <v>1</v>
-      </c>
-      <c r="L52" t="n">
-        <v>1</v>
-      </c>
       <c r="M52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N52" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" t="n">
+        <v>3</v>
+      </c>
+      <c r="P52" t="n">
         <v>4</v>
       </c>
-      <c r="O52" t="n">
+      <c r="Q52" t="n">
         <v>4</v>
       </c>
-      <c r="P52" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>1</v>
-      </c>
-      <c r="X52" t="n">
+      <c r="R52" t="n">
+        <v>2</v>
+      </c>
+      <c r="S52" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z52" t="n">
         <v>15</v>
       </c>
-      <c r="Y52" t="n">
+      <c r="AA52" t="n">
         <v>2388.75</v>
       </c>
     </row>
@@ -3634,34 +3932,36 @@
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
       <c r="I53" s="2" t="n"/>
-      <c r="J53" t="n">
+      <c r="J53" s="2" t="n"/>
+      <c r="K53" s="2" t="n"/>
+      <c r="L53" t="n">
         <v>161.58</v>
       </c>
-      <c r="K53" t="n">
-        <v>1</v>
-      </c>
-      <c r="L53" t="n">
-        <v>1</v>
-      </c>
       <c r="M53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N53" t="n">
+        <v>1</v>
+      </c>
+      <c r="O53" t="n">
+        <v>3</v>
+      </c>
+      <c r="P53" t="n">
         <v>4</v>
       </c>
-      <c r="O53" t="n">
+      <c r="Q53" t="n">
         <v>4</v>
       </c>
-      <c r="P53" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>1</v>
-      </c>
-      <c r="X53" t="n">
+      <c r="R53" t="n">
+        <v>2</v>
+      </c>
+      <c r="S53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z53" t="n">
         <v>15</v>
       </c>
-      <c r="Y53" t="n">
+      <c r="AA53" t="n">
         <v>2423.7</v>
       </c>
     </row>
@@ -3695,37 +3995,39 @@
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
-      <c r="J54" t="n">
+      <c r="J54" s="2" t="n"/>
+      <c r="K54" s="2" t="n"/>
+      <c r="L54" t="n">
         <v>135.3</v>
       </c>
-      <c r="K54" t="n">
-        <v>1</v>
-      </c>
-      <c r="P54" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>3</v>
+      <c r="M54" t="n">
+        <v>1</v>
       </c>
       <c r="R54" t="n">
+        <v>1</v>
+      </c>
+      <c r="S54" t="n">
+        <v>3</v>
+      </c>
+      <c r="T54" t="n">
         <v>4</v>
       </c>
-      <c r="S54" t="n">
+      <c r="U54" t="n">
         <v>4</v>
       </c>
-      <c r="T54" t="n">
-        <v>3</v>
-      </c>
-      <c r="U54" t="n">
-        <v>2</v>
-      </c>
       <c r="V54" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="W54" t="n">
+        <v>2</v>
       </c>
       <c r="X54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z54" t="n">
         <v>18</v>
       </c>
-      <c r="Y54" t="n">
+      <c r="AA54" t="n">
         <v>2435.4</v>
       </c>
     </row>
@@ -3772,36 +4074,44 @@
         </is>
       </c>
       <c r="J55" t="n">
+        <v>439.9</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
         <v>153.55</v>
       </c>
-      <c r="K55" t="n">
-        <v>1</v>
-      </c>
-      <c r="P55" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>3</v>
+      <c r="M55" t="n">
+        <v>1</v>
       </c>
       <c r="R55" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S55" t="n">
         <v>3</v>
       </c>
       <c r="T55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V55" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="W55" t="n">
+        <v>2</v>
       </c>
       <c r="X55" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z55" t="n">
         <v>15</v>
       </c>
-      <c r="Y55" t="n">
+      <c r="AA55" t="n">
         <v>2303.25</v>
       </c>
     </row>
@@ -3835,37 +4145,39 @@
       <c r="G56" s="2" t="n"/>
       <c r="H56" s="2" t="n"/>
       <c r="I56" s="2" t="n"/>
-      <c r="J56" t="n">
+      <c r="J56" s="2" t="n"/>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" t="n">
         <v>159.78</v>
       </c>
-      <c r="K56" t="n">
-        <v>1</v>
-      </c>
-      <c r="P56" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q56" t="n">
-        <v>3</v>
+      <c r="M56" t="n">
+        <v>1</v>
       </c>
       <c r="R56" t="n">
+        <v>1</v>
+      </c>
+      <c r="S56" t="n">
+        <v>3</v>
+      </c>
+      <c r="T56" t="n">
         <v>4</v>
       </c>
-      <c r="S56" t="n">
+      <c r="U56" t="n">
         <v>4</v>
       </c>
-      <c r="T56" t="n">
-        <v>3</v>
-      </c>
-      <c r="U56" t="n">
-        <v>2</v>
-      </c>
       <c r="V56" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="W56" t="n">
+        <v>2</v>
       </c>
       <c r="X56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z56" t="n">
         <v>18</v>
       </c>
-      <c r="Y56" t="n">
+      <c r="AA56" t="n">
         <v>2876.04</v>
       </c>
     </row>
@@ -3912,30 +4224,38 @@
         </is>
       </c>
       <c r="J57" t="n">
+        <v>439.9</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
         <v>145.11</v>
       </c>
-      <c r="K57" t="n">
-        <v>1</v>
-      </c>
-      <c r="P57" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q57" t="n">
-        <v>2</v>
+      <c r="M57" t="n">
+        <v>1</v>
       </c>
       <c r="R57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T57" t="n">
         <v>3</v>
       </c>
-      <c r="X57" t="n">
+      <c r="U57" t="n">
+        <v>3</v>
+      </c>
+      <c r="V57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z57" t="n">
         <v>12</v>
       </c>
-      <c r="Y57" t="n">
+      <c r="AA57" t="n">
         <v>1741.32</v>
       </c>
     </row>
@@ -3982,33 +4302,41 @@
         </is>
       </c>
       <c r="J58" t="n">
+        <v>399.9</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
         <v>138.2</v>
       </c>
-      <c r="K58" t="n">
-        <v>1</v>
-      </c>
-      <c r="L58" t="n">
-        <v>1</v>
-      </c>
       <c r="M58" t="n">
         <v>1</v>
       </c>
       <c r="N58" t="n">
+        <v>1</v>
+      </c>
+      <c r="O58" t="n">
+        <v>1</v>
+      </c>
+      <c r="P58" t="n">
         <v>4</v>
       </c>
-      <c r="O58" t="n">
+      <c r="Q58" t="n">
         <v>5</v>
       </c>
-      <c r="P58" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q58" t="n">
-        <v>1</v>
-      </c>
-      <c r="X58" t="n">
+      <c r="R58" t="n">
+        <v>3</v>
+      </c>
+      <c r="S58" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z58" t="n">
         <v>15</v>
       </c>
-      <c r="Y58" t="n">
+      <c r="AA58" t="n">
         <v>2073</v>
       </c>
     </row>
@@ -4055,18 +4383,26 @@
         </is>
       </c>
       <c r="J59" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
         <v>52.89</v>
       </c>
-      <c r="K59" t="n">
-        <v>1</v>
-      </c>
-      <c r="W59" t="n">
+      <c r="M59" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y59" t="n">
         <v>9</v>
       </c>
-      <c r="X59" t="n">
+      <c r="Z59" t="n">
         <v>9</v>
       </c>
-      <c r="Y59" t="n">
+      <c r="AA59" t="n">
         <v>476.01</v>
       </c>
     </row>
@@ -4113,18 +4449,26 @@
         </is>
       </c>
       <c r="J60" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
         <v>52.89</v>
       </c>
-      <c r="K60" t="n">
-        <v>1</v>
-      </c>
-      <c r="W60" t="n">
+      <c r="M60" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y60" t="n">
         <v>6</v>
       </c>
-      <c r="X60" t="n">
+      <c r="Z60" t="n">
         <v>6</v>
       </c>
-      <c r="Y60" t="n">
+      <c r="AA60" t="n">
         <v>317.34</v>
       </c>
     </row>
@@ -4171,18 +4515,26 @@
         </is>
       </c>
       <c r="J61" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L61" t="n">
         <v>39.04</v>
       </c>
-      <c r="K61" t="n">
-        <v>1</v>
-      </c>
-      <c r="W61" t="n">
+      <c r="M61" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y61" t="n">
         <v>9</v>
       </c>
-      <c r="X61" t="n">
+      <c r="Z61" t="n">
         <v>9</v>
       </c>
-      <c r="Y61" t="n">
+      <c r="AA61" t="n">
         <v>351.36</v>
       </c>
     </row>
@@ -4229,18 +4581,26 @@
         </is>
       </c>
       <c r="J62" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L62" t="n">
         <v>39.04</v>
       </c>
-      <c r="K62" t="n">
-        <v>1</v>
-      </c>
-      <c r="W62" t="n">
+      <c r="M62" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y62" t="n">
         <v>9</v>
       </c>
-      <c r="X62" t="n">
+      <c r="Z62" t="n">
         <v>9</v>
       </c>
-      <c r="Y62" t="n">
+      <c r="AA62" t="n">
         <v>351.36</v>
       </c>
     </row>
@@ -4287,33 +4647,41 @@
         </is>
       </c>
       <c r="J63" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
         <v>61.13</v>
       </c>
-      <c r="K63" t="n">
-        <v>1</v>
-      </c>
-      <c r="L63" t="n">
-        <v>1</v>
-      </c>
       <c r="M63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N63" t="n">
+        <v>1</v>
+      </c>
+      <c r="O63" t="n">
+        <v>3</v>
+      </c>
+      <c r="P63" t="n">
         <v>4</v>
       </c>
-      <c r="O63" t="n">
-        <v>3</v>
-      </c>
-      <c r="P63" t="n">
-        <v>3</v>
-      </c>
       <c r="Q63" t="n">
-        <v>1</v>
-      </c>
-      <c r="X63" t="n">
+        <v>3</v>
+      </c>
+      <c r="R63" t="n">
+        <v>3</v>
+      </c>
+      <c r="S63" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z63" t="n">
         <v>15</v>
       </c>
-      <c r="Y63" t="n">
+      <c r="AA63" t="n">
         <v>916.95</v>
       </c>
     </row>
@@ -4347,34 +4715,36 @@
       <c r="G64" s="2" t="n"/>
       <c r="H64" s="2" t="n"/>
       <c r="I64" s="2" t="n"/>
-      <c r="J64" t="n">
+      <c r="J64" s="2" t="n"/>
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" t="n">
         <v>70.93000000000001</v>
       </c>
-      <c r="K64" t="n">
-        <v>1</v>
-      </c>
-      <c r="L64" t="n">
-        <v>1</v>
-      </c>
       <c r="M64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N64" t="n">
+        <v>1</v>
+      </c>
+      <c r="O64" t="n">
+        <v>3</v>
+      </c>
+      <c r="P64" t="n">
         <v>4</v>
       </c>
-      <c r="O64" t="n">
-        <v>3</v>
-      </c>
-      <c r="P64" t="n">
-        <v>3</v>
-      </c>
       <c r="Q64" t="n">
-        <v>1</v>
-      </c>
-      <c r="X64" t="n">
+        <v>3</v>
+      </c>
+      <c r="R64" t="n">
+        <v>3</v>
+      </c>
+      <c r="S64" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z64" t="n">
         <v>15</v>
       </c>
-      <c r="Y64" t="n">
+      <c r="AA64" t="n">
         <v>1063.95</v>
       </c>
     </row>
@@ -4408,34 +4778,36 @@
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n"/>
       <c r="I65" s="2" t="n"/>
-      <c r="J65" t="n">
+      <c r="J65" s="2" t="n"/>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" t="n">
         <v>70.93000000000001</v>
       </c>
-      <c r="K65" t="n">
-        <v>1</v>
-      </c>
-      <c r="L65" t="n">
-        <v>1</v>
-      </c>
       <c r="M65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q65" t="n">
-        <v>1</v>
-      </c>
-      <c r="X65" t="n">
+        <v>3</v>
+      </c>
+      <c r="R65" t="n">
+        <v>2</v>
+      </c>
+      <c r="S65" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z65" t="n">
         <v>12</v>
       </c>
-      <c r="Y65" t="n">
+      <c r="AA65" t="n">
         <v>851.16</v>
       </c>
     </row>
@@ -4469,34 +4841,36 @@
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="n"/>
-      <c r="J66" t="n">
+      <c r="J66" s="2" t="n"/>
+      <c r="K66" s="2" t="n"/>
+      <c r="L66" t="n">
         <v>56.96</v>
       </c>
-      <c r="K66" t="n">
-        <v>1</v>
-      </c>
-      <c r="L66" t="n">
-        <v>1</v>
-      </c>
       <c r="M66" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N66" t="n">
+        <v>1</v>
+      </c>
+      <c r="O66" t="n">
+        <v>3</v>
+      </c>
+      <c r="P66" t="n">
         <v>5</v>
       </c>
-      <c r="O66" t="n">
+      <c r="Q66" t="n">
         <v>4</v>
       </c>
-      <c r="P66" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q66" t="n">
-        <v>2</v>
-      </c>
-      <c r="X66" t="n">
+      <c r="R66" t="n">
+        <v>3</v>
+      </c>
+      <c r="S66" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z66" t="n">
         <v>18</v>
       </c>
-      <c r="Y66" t="n">
+      <c r="AA66" t="n">
         <v>1025.28</v>
       </c>
     </row>

</xml_diff>